<commit_message>
new rows to il_courts.xlsx
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/il_courts.xlsx
+++ b/docassemble/ILAO/data/sources/il_courts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VivianM\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\local-DA-easyforms-dev\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BD88A19-40BE-49BE-B6A5-DC1B764F7A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3866A7E-5F96-4F20-9E44-E29745CE2B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="770">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1163" uniqueCount="783">
   <si>
     <t>court_code</t>
   </si>
@@ -2335,6 +2335,45 @@
   </si>
   <si>
     <t>https://24thcircuit.illinoiscourts.gov/</t>
+  </si>
+  <si>
+    <t>Kane County Judicial Center</t>
+  </si>
+  <si>
+    <t>37W777 Route 38</t>
+  </si>
+  <si>
+    <t>St. Charles</t>
+  </si>
+  <si>
+    <t>Kane County Juvenile Justice Center</t>
+  </si>
+  <si>
+    <t>37W655 Route 38</t>
+  </si>
+  <si>
+    <t>530 S. Randall Road</t>
+  </si>
+  <si>
+    <t>Aurora Branch Court</t>
+  </si>
+  <si>
+    <t>1200 East Indian Trail Road</t>
+  </si>
+  <si>
+    <t>Aurora</t>
+  </si>
+  <si>
+    <t>Elgin</t>
+  </si>
+  <si>
+    <t>Elgin Branch Court</t>
+  </si>
+  <si>
+    <t>150 Dexter Court</t>
+  </si>
+  <si>
+    <t>Kane County Branch Court</t>
   </si>
 </sst>
 </file>
@@ -2786,14 +2825,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V111"/>
+  <dimension ref="A1:V116"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" customWidth="1"/>
     <col min="2" max="2" width="36.109375" customWidth="1"/>
     <col min="3" max="3" width="10.44140625" customWidth="1"/>
-    <col min="4" max="4" width="2.77734375" customWidth="1"/>
-    <col min="5" max="5" width="3" customWidth="1"/>
+    <col min="4" max="4" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="2.109375" customWidth="1"/>
     <col min="7" max="7" width="2.33203125" customWidth="1"/>
     <col min="8" max="8" width="13.6640625" customWidth="1"/>
@@ -4897,759 +4936,759 @@
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>46</v>
+        <v>111</v>
       </c>
       <c r="B55" t="s">
-        <v>377</v>
+        <v>770</v>
       </c>
       <c r="C55" t="s">
         <v>23</v>
       </c>
       <c r="H55" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
       <c r="K55" t="s">
-        <v>379</v>
+        <v>771</v>
       </c>
       <c r="M55" t="s">
-        <v>380</v>
+        <v>772</v>
       </c>
       <c r="N55" t="s">
         <v>27</v>
       </c>
       <c r="O55">
-        <v>60901</v>
+        <v>60175</v>
       </c>
       <c r="P55" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="Q55" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="R55" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="V55" t="s">
-        <v>330</v>
+        <v>376</v>
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="B56" t="s">
-        <v>383</v>
+        <v>773</v>
       </c>
       <c r="C56" t="s">
         <v>23</v>
       </c>
       <c r="H56" t="s">
-        <v>384</v>
+        <v>370</v>
       </c>
       <c r="K56" t="s">
-        <v>385</v>
+        <v>774</v>
       </c>
       <c r="M56" t="s">
-        <v>386</v>
+        <v>772</v>
       </c>
       <c r="N56" t="s">
         <v>27</v>
       </c>
       <c r="O56">
-        <v>60560</v>
+        <v>60174</v>
       </c>
       <c r="P56" t="s">
-        <v>387</v>
+        <v>373</v>
       </c>
       <c r="Q56" t="s">
-        <v>388</v>
+        <v>374</v>
       </c>
       <c r="R56" t="s">
-        <v>389</v>
+        <v>375</v>
       </c>
       <c r="V56" t="s">
-        <v>200</v>
+        <v>376</v>
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>48</v>
+        <v>113</v>
       </c>
       <c r="B57" t="s">
-        <v>390</v>
+        <v>782</v>
       </c>
       <c r="C57" t="s">
         <v>23</v>
       </c>
       <c r="H57" t="s">
-        <v>391</v>
+        <v>370</v>
       </c>
       <c r="K57" t="s">
-        <v>392</v>
+        <v>775</v>
       </c>
       <c r="M57" t="s">
-        <v>393</v>
+        <v>772</v>
       </c>
       <c r="N57" t="s">
         <v>27</v>
       </c>
       <c r="O57">
-        <v>61401</v>
+        <v>60174</v>
       </c>
       <c r="P57" t="s">
-        <v>394</v>
+        <v>373</v>
       </c>
       <c r="Q57" t="s">
-        <v>395</v>
+        <v>374</v>
       </c>
       <c r="R57" t="s">
-        <v>396</v>
+        <v>375</v>
       </c>
       <c r="V57" t="s">
-        <v>270</v>
+        <v>376</v>
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A58">
-        <v>49</v>
+        <v>114</v>
       </c>
       <c r="B58" t="s">
-        <v>397</v>
+        <v>776</v>
       </c>
       <c r="C58" t="s">
         <v>23</v>
       </c>
       <c r="H58" t="s">
-        <v>398</v>
+        <v>370</v>
       </c>
       <c r="K58" t="s">
-        <v>399</v>
+        <v>777</v>
       </c>
       <c r="M58" t="s">
-        <v>400</v>
+        <v>778</v>
       </c>
       <c r="N58" t="s">
         <v>27</v>
       </c>
       <c r="O58">
-        <v>60085</v>
+        <v>60505</v>
       </c>
       <c r="P58" t="s">
-        <v>401</v>
+        <v>373</v>
       </c>
       <c r="Q58" t="s">
-        <v>402</v>
+        <v>374</v>
       </c>
       <c r="R58" t="s">
-        <v>403</v>
+        <v>375</v>
       </c>
       <c r="V58" t="s">
-        <v>404</v>
+        <v>376</v>
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>50</v>
+        <v>115</v>
       </c>
       <c r="B59" t="s">
-        <v>405</v>
+        <v>780</v>
       </c>
       <c r="C59" t="s">
         <v>23</v>
       </c>
       <c r="H59" t="s">
-        <v>406</v>
+        <v>370</v>
       </c>
       <c r="K59" t="s">
-        <v>407</v>
+        <v>781</v>
       </c>
       <c r="M59" t="s">
-        <v>408</v>
+        <v>779</v>
       </c>
       <c r="N59" t="s">
         <v>27</v>
       </c>
       <c r="O59">
-        <v>61350</v>
+        <v>60120</v>
       </c>
       <c r="P59" t="s">
-        <v>409</v>
+        <v>373</v>
       </c>
       <c r="Q59" t="s">
-        <v>410</v>
+        <v>374</v>
       </c>
       <c r="R59" t="s">
-        <v>411</v>
+        <v>375</v>
       </c>
       <c r="V59" t="s">
-        <v>70</v>
+        <v>376</v>
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B60" t="s">
-        <v>412</v>
+        <v>377</v>
       </c>
       <c r="C60" t="s">
         <v>23</v>
       </c>
       <c r="H60" t="s">
-        <v>413</v>
+        <v>378</v>
       </c>
       <c r="K60" t="s">
-        <v>414</v>
+        <v>379</v>
       </c>
       <c r="M60" t="s">
-        <v>415</v>
+        <v>380</v>
       </c>
       <c r="N60" t="s">
         <v>27</v>
       </c>
       <c r="O60">
-        <v>62439</v>
+        <v>60901</v>
       </c>
       <c r="P60" t="s">
-        <v>416</v>
-      </c>
-      <c r="Q60" s="2" t="s">
-        <v>767</v>
+        <v>380</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>381</v>
       </c>
       <c r="R60" t="s">
-        <v>417</v>
+        <v>382</v>
       </c>
       <c r="V60" t="s">
-        <v>185</v>
+        <v>330</v>
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B61" t="s">
-        <v>418</v>
+        <v>383</v>
       </c>
       <c r="C61" t="s">
         <v>23</v>
       </c>
       <c r="H61" t="s">
-        <v>419</v>
+        <v>384</v>
       </c>
       <c r="K61" t="s">
-        <v>420</v>
+        <v>385</v>
       </c>
       <c r="M61" t="s">
-        <v>421</v>
+        <v>386</v>
       </c>
       <c r="N61" t="s">
         <v>27</v>
       </c>
       <c r="O61">
-        <v>61021</v>
+        <v>60560</v>
       </c>
       <c r="P61" t="s">
-        <v>422</v>
+        <v>387</v>
       </c>
       <c r="Q61" t="s">
-        <v>423</v>
+        <v>388</v>
       </c>
       <c r="R61" t="s">
-        <v>424</v>
+        <v>389</v>
       </c>
       <c r="V61" t="s">
-        <v>425</v>
+        <v>200</v>
       </c>
     </row>
     <row r="62" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B62" t="s">
-        <v>426</v>
+        <v>390</v>
       </c>
       <c r="C62" t="s">
         <v>23</v>
       </c>
       <c r="H62" t="s">
-        <v>427</v>
+        <v>391</v>
       </c>
       <c r="K62" t="s">
-        <v>428</v>
+        <v>392</v>
       </c>
       <c r="M62" t="s">
-        <v>429</v>
+        <v>393</v>
       </c>
       <c r="N62" t="s">
         <v>27</v>
       </c>
       <c r="O62">
-        <v>61764</v>
+        <v>61401</v>
       </c>
       <c r="P62" t="s">
-        <v>430</v>
+        <v>394</v>
       </c>
       <c r="Q62" t="s">
-        <v>431</v>
+        <v>395</v>
       </c>
       <c r="R62" t="s">
-        <v>432</v>
+        <v>396</v>
       </c>
       <c r="V62" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
     </row>
     <row r="63" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B63" t="s">
-        <v>433</v>
+        <v>397</v>
       </c>
       <c r="C63" t="s">
         <v>23</v>
       </c>
       <c r="H63" t="s">
-        <v>434</v>
+        <v>398</v>
       </c>
       <c r="K63" t="s">
-        <v>435</v>
+        <v>399</v>
       </c>
       <c r="M63" t="s">
-        <v>436</v>
+        <v>400</v>
       </c>
       <c r="N63" t="s">
         <v>27</v>
       </c>
       <c r="O63">
-        <v>62656</v>
+        <v>60085</v>
       </c>
       <c r="P63" t="s">
-        <v>437</v>
+        <v>401</v>
       </c>
       <c r="Q63" t="s">
-        <v>438</v>
+        <v>402</v>
       </c>
       <c r="R63" t="s">
-        <v>439</v>
+        <v>403</v>
       </c>
       <c r="V63" t="s">
-        <v>255</v>
+        <v>404</v>
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A64">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B64" t="s">
-        <v>440</v>
+        <v>405</v>
       </c>
       <c r="C64" t="s">
         <v>23</v>
       </c>
       <c r="H64" t="s">
-        <v>441</v>
+        <v>406</v>
       </c>
       <c r="K64" t="s">
-        <v>442</v>
+        <v>407</v>
       </c>
       <c r="M64" t="s">
-        <v>443</v>
+        <v>408</v>
       </c>
       <c r="N64" t="s">
         <v>27</v>
       </c>
       <c r="O64">
-        <v>62523</v>
+        <v>61350</v>
       </c>
       <c r="P64" t="s">
-        <v>444</v>
+        <v>409</v>
       </c>
       <c r="Q64" t="s">
-        <v>445</v>
+        <v>410</v>
       </c>
       <c r="R64" t="s">
-        <v>446</v>
+        <v>411</v>
       </c>
       <c r="V64" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B65" t="s">
-        <v>447</v>
+        <v>412</v>
       </c>
       <c r="C65" t="s">
         <v>23</v>
       </c>
       <c r="H65" t="s">
-        <v>448</v>
+        <v>413</v>
       </c>
       <c r="K65" t="s">
-        <v>449</v>
+        <v>414</v>
       </c>
       <c r="M65" t="s">
-        <v>450</v>
+        <v>415</v>
       </c>
       <c r="N65" t="s">
         <v>27</v>
       </c>
       <c r="O65">
-        <v>62626</v>
+        <v>62439</v>
       </c>
       <c r="P65" t="s">
-        <v>451</v>
-      </c>
-      <c r="Q65" t="s">
-        <v>452</v>
+        <v>416</v>
+      </c>
+      <c r="Q65" s="2" t="s">
+        <v>767</v>
       </c>
       <c r="R65" t="s">
-        <v>453</v>
+        <v>417</v>
       </c>
       <c r="V65" t="s">
-        <v>283</v>
+        <v>185</v>
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B66" t="s">
-        <v>454</v>
+        <v>418</v>
       </c>
       <c r="C66" t="s">
         <v>23</v>
       </c>
       <c r="H66" t="s">
-        <v>455</v>
+        <v>419</v>
       </c>
       <c r="K66" t="s">
-        <v>456</v>
+        <v>420</v>
       </c>
       <c r="M66" t="s">
-        <v>457</v>
+        <v>421</v>
       </c>
       <c r="N66" t="s">
         <v>27</v>
       </c>
       <c r="O66">
-        <v>62025</v>
+        <v>61021</v>
       </c>
       <c r="P66" t="s">
-        <v>458</v>
+        <v>422</v>
       </c>
       <c r="Q66" t="s">
-        <v>459</v>
+        <v>423</v>
       </c>
       <c r="R66" t="s">
-        <v>460</v>
+        <v>424</v>
       </c>
       <c r="V66" t="s">
-        <v>47</v>
+        <v>425</v>
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B67" t="s">
-        <v>461</v>
+        <v>426</v>
       </c>
       <c r="C67" t="s">
         <v>23</v>
       </c>
       <c r="H67" t="s">
-        <v>462</v>
+        <v>427</v>
       </c>
       <c r="K67" t="s">
-        <v>463</v>
+        <v>428</v>
       </c>
       <c r="M67" t="s">
-        <v>464</v>
+        <v>429</v>
       </c>
       <c r="N67" t="s">
         <v>27</v>
       </c>
       <c r="O67">
-        <v>62881</v>
+        <v>61764</v>
       </c>
       <c r="P67" t="s">
-        <v>465</v>
+        <v>430</v>
       </c>
       <c r="Q67" t="s">
-        <v>466</v>
+        <v>431</v>
       </c>
       <c r="R67" t="s">
-        <v>467</v>
+        <v>432</v>
       </c>
       <c r="V67" t="s">
-        <v>108</v>
+        <v>255</v>
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B68" t="s">
-        <v>468</v>
+        <v>433</v>
       </c>
       <c r="C68" t="s">
         <v>23</v>
       </c>
       <c r="H68" t="s">
-        <v>469</v>
+        <v>434</v>
       </c>
       <c r="K68" t="s">
-        <v>470</v>
+        <v>435</v>
       </c>
       <c r="M68" t="s">
-        <v>471</v>
+        <v>436</v>
       </c>
       <c r="N68" t="s">
         <v>27</v>
       </c>
       <c r="O68">
-        <v>61540</v>
+        <v>62656</v>
       </c>
       <c r="P68" t="s">
-        <v>112</v>
+        <v>437</v>
       </c>
       <c r="Q68" t="s">
-        <v>472</v>
+        <v>438</v>
       </c>
       <c r="R68" t="s">
-        <v>473</v>
+        <v>439</v>
       </c>
       <c r="V68" t="s">
-        <v>474</v>
+        <v>255</v>
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A69">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B69" t="s">
-        <v>475</v>
+        <v>440</v>
       </c>
       <c r="C69" t="s">
         <v>23</v>
       </c>
       <c r="H69" t="s">
-        <v>476</v>
+        <v>441</v>
       </c>
       <c r="K69" t="s">
-        <v>477</v>
+        <v>442</v>
       </c>
       <c r="M69" t="s">
-        <v>478</v>
+        <v>443</v>
       </c>
       <c r="N69" t="s">
         <v>27</v>
       </c>
       <c r="O69">
-        <v>62644</v>
+        <v>62523</v>
       </c>
       <c r="P69" t="s">
-        <v>479</v>
+        <v>444</v>
       </c>
       <c r="Q69" t="s">
-        <v>480</v>
+        <v>445</v>
       </c>
       <c r="R69" t="s">
-        <v>481</v>
+        <v>446</v>
       </c>
       <c r="V69" t="s">
-        <v>31</v>
+        <v>100</v>
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A70">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B70" t="s">
-        <v>482</v>
+        <v>447</v>
       </c>
       <c r="C70" t="s">
         <v>23</v>
       </c>
       <c r="H70" t="s">
-        <v>483</v>
+        <v>448</v>
       </c>
       <c r="K70" t="s">
-        <v>484</v>
+        <v>449</v>
       </c>
       <c r="M70" t="s">
-        <v>485</v>
+        <v>450</v>
       </c>
       <c r="N70" t="s">
         <v>27</v>
       </c>
       <c r="O70">
-        <v>62960</v>
+        <v>62626</v>
       </c>
       <c r="P70" t="s">
-        <v>486</v>
+        <v>451</v>
       </c>
       <c r="Q70" t="s">
-        <v>37</v>
+        <v>452</v>
       </c>
       <c r="R70" t="s">
-        <v>487</v>
+        <v>453</v>
       </c>
       <c r="V70" t="s">
-        <v>39</v>
+        <v>283</v>
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A71">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B71" t="s">
-        <v>488</v>
+        <v>454</v>
       </c>
       <c r="C71" t="s">
         <v>23</v>
       </c>
       <c r="H71" t="s">
-        <v>489</v>
+        <v>455</v>
       </c>
       <c r="K71" t="s">
-        <v>490</v>
+        <v>456</v>
       </c>
       <c r="M71" t="s">
-        <v>491</v>
+        <v>457</v>
       </c>
       <c r="N71" t="s">
         <v>27</v>
       </c>
       <c r="O71">
-        <v>61455</v>
+        <v>62025</v>
       </c>
       <c r="P71" t="s">
-        <v>492</v>
+        <v>458</v>
       </c>
       <c r="Q71" t="s">
-        <v>493</v>
+        <v>459</v>
       </c>
       <c r="R71" t="s">
-        <v>494</v>
+        <v>460</v>
       </c>
       <c r="V71" t="s">
-        <v>270</v>
+        <v>47</v>
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A72">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B72" t="s">
-        <v>495</v>
+        <v>461</v>
       </c>
       <c r="C72" t="s">
         <v>23</v>
       </c>
       <c r="H72" t="s">
-        <v>496</v>
+        <v>462</v>
       </c>
       <c r="K72" t="s">
-        <v>497</v>
+        <v>463</v>
       </c>
       <c r="M72" t="s">
-        <v>498</v>
+        <v>464</v>
       </c>
       <c r="N72" t="s">
         <v>27</v>
       </c>
       <c r="O72">
-        <v>60098</v>
+        <v>62881</v>
       </c>
       <c r="P72" t="s">
-        <v>499</v>
+        <v>465</v>
       </c>
       <c r="Q72" t="s">
-        <v>500</v>
+        <v>466</v>
       </c>
       <c r="R72" t="s">
-        <v>501</v>
+        <v>467</v>
       </c>
       <c r="V72" t="s">
-        <v>502</v>
+        <v>108</v>
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A73">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B73" t="s">
-        <v>503</v>
+        <v>468</v>
       </c>
       <c r="C73" t="s">
         <v>23</v>
       </c>
       <c r="H73" t="s">
-        <v>504</v>
+        <v>469</v>
       </c>
       <c r="K73" t="s">
-        <v>505</v>
+        <v>470</v>
       </c>
       <c r="M73" t="s">
-        <v>506</v>
+        <v>471</v>
       </c>
       <c r="N73" t="s">
         <v>27</v>
       </c>
       <c r="O73">
-        <v>61701</v>
+        <v>61540</v>
       </c>
       <c r="P73" t="s">
-        <v>507</v>
+        <v>112</v>
       </c>
       <c r="Q73" t="s">
-        <v>508</v>
+        <v>472</v>
       </c>
       <c r="R73" t="s">
-        <v>509</v>
+        <v>473</v>
       </c>
       <c r="V73" t="s">
-        <v>255</v>
+        <v>474</v>
       </c>
     </row>
     <row r="74" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A74">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B74" t="s">
-        <v>510</v>
+        <v>475</v>
       </c>
       <c r="C74" t="s">
         <v>23</v>
       </c>
       <c r="H74" t="s">
-        <v>511</v>
+        <v>476</v>
       </c>
       <c r="K74" t="s">
-        <v>512</v>
+        <v>477</v>
       </c>
       <c r="M74" t="s">
-        <v>513</v>
+        <v>478</v>
       </c>
       <c r="N74" t="s">
         <v>27</v>
       </c>
       <c r="O74">
-        <v>62675</v>
+        <v>62644</v>
       </c>
       <c r="P74" t="s">
-        <v>514</v>
+        <v>479</v>
       </c>
       <c r="Q74" t="s">
-        <v>515</v>
+        <v>480</v>
       </c>
       <c r="R74" t="s">
-        <v>516</v>
+        <v>481</v>
       </c>
       <c r="V74" t="s">
         <v>31</v>
@@ -5657,645 +5696,645 @@
     </row>
     <row r="75" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A75">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B75" t="s">
-        <v>517</v>
+        <v>482</v>
       </c>
       <c r="C75" t="s">
         <v>23</v>
       </c>
       <c r="H75" t="s">
-        <v>518</v>
+        <v>483</v>
       </c>
       <c r="K75" t="s">
-        <v>519</v>
+        <v>484</v>
       </c>
       <c r="M75" t="s">
-        <v>520</v>
+        <v>485</v>
       </c>
       <c r="N75" t="s">
         <v>27</v>
       </c>
       <c r="O75">
-        <v>61231</v>
+        <v>62960</v>
       </c>
       <c r="P75" t="s">
-        <v>521</v>
+        <v>486</v>
       </c>
       <c r="Q75" t="s">
-        <v>522</v>
+        <v>37</v>
       </c>
       <c r="R75" t="s">
-        <v>523</v>
+        <v>487</v>
       </c>
       <c r="V75" t="s">
-        <v>322</v>
+        <v>39</v>
       </c>
     </row>
     <row r="76" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A76">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B76" t="s">
-        <v>524</v>
+        <v>488</v>
       </c>
       <c r="C76" t="s">
         <v>23</v>
       </c>
       <c r="H76" t="s">
-        <v>525</v>
+        <v>489</v>
       </c>
       <c r="K76" t="s">
-        <v>526</v>
+        <v>490</v>
       </c>
       <c r="M76" t="s">
-        <v>527</v>
+        <v>491</v>
       </c>
       <c r="N76" t="s">
         <v>27</v>
       </c>
       <c r="O76">
-        <v>62298</v>
+        <v>61455</v>
       </c>
       <c r="P76" t="s">
-        <v>528</v>
+        <v>492</v>
       </c>
       <c r="Q76" t="s">
-        <v>529</v>
+        <v>493</v>
       </c>
       <c r="R76" t="s">
-        <v>530</v>
+        <v>494</v>
       </c>
       <c r="V76" t="s">
-        <v>531</v>
+        <v>270</v>
       </c>
     </row>
     <row r="77" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A77">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B77" t="s">
-        <v>532</v>
+        <v>495</v>
       </c>
       <c r="C77" t="s">
         <v>23</v>
       </c>
       <c r="H77" t="s">
-        <v>533</v>
+        <v>496</v>
       </c>
       <c r="K77" t="s">
-        <v>534</v>
+        <v>497</v>
       </c>
       <c r="M77" t="s">
-        <v>535</v>
+        <v>498</v>
       </c>
       <c r="N77" t="s">
         <v>27</v>
       </c>
       <c r="O77">
-        <v>62049</v>
+        <v>60098</v>
       </c>
       <c r="P77" t="s">
-        <v>536</v>
+        <v>499</v>
       </c>
       <c r="Q77" t="s">
-        <v>537</v>
+        <v>500</v>
       </c>
       <c r="R77" t="s">
-        <v>538</v>
+        <v>501</v>
       </c>
       <c r="V77" t="s">
-        <v>108</v>
+        <v>502</v>
       </c>
     </row>
     <row r="78" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A78">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B78" t="s">
-        <v>539</v>
+        <v>503</v>
       </c>
       <c r="C78" t="s">
         <v>23</v>
       </c>
       <c r="H78" t="s">
-        <v>540</v>
+        <v>504</v>
       </c>
       <c r="K78" t="s">
-        <v>541</v>
+        <v>505</v>
       </c>
       <c r="M78" t="s">
-        <v>542</v>
+        <v>506</v>
       </c>
       <c r="N78" t="s">
         <v>27</v>
       </c>
       <c r="O78">
-        <v>62650</v>
+        <v>61701</v>
       </c>
       <c r="P78" t="s">
-        <v>543</v>
+        <v>507</v>
       </c>
       <c r="Q78" t="s">
-        <v>544</v>
+        <v>508</v>
       </c>
       <c r="R78" t="s">
-        <v>545</v>
+        <v>509</v>
       </c>
       <c r="V78" t="s">
-        <v>283</v>
+        <v>255</v>
       </c>
     </row>
     <row r="79" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A79">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B79" t="s">
-        <v>546</v>
+        <v>510</v>
       </c>
       <c r="C79" t="s">
         <v>23</v>
       </c>
       <c r="H79" t="s">
-        <v>547</v>
+        <v>511</v>
       </c>
       <c r="K79" t="s">
-        <v>548</v>
+        <v>512</v>
       </c>
       <c r="M79" t="s">
-        <v>549</v>
+        <v>513</v>
       </c>
       <c r="N79" t="s">
         <v>27</v>
       </c>
       <c r="O79">
-        <v>61951</v>
+        <v>62675</v>
       </c>
       <c r="P79" t="s">
-        <v>550</v>
+        <v>514</v>
       </c>
       <c r="Q79" t="s">
-        <v>551</v>
+        <v>515</v>
       </c>
       <c r="R79" t="s">
-        <v>552</v>
+        <v>516</v>
       </c>
       <c r="V79" t="s">
-        <v>100</v>
+        <v>31</v>
       </c>
     </row>
     <row r="80" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A80">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B80" t="s">
-        <v>553</v>
+        <v>517</v>
       </c>
       <c r="C80" t="s">
         <v>23</v>
       </c>
       <c r="H80" t="s">
-        <v>554</v>
+        <v>518</v>
       </c>
       <c r="K80" t="s">
-        <v>555</v>
+        <v>519</v>
       </c>
       <c r="M80" t="s">
-        <v>556</v>
+        <v>520</v>
       </c>
       <c r="N80" t="s">
         <v>27</v>
       </c>
       <c r="O80">
-        <v>61061</v>
+        <v>61231</v>
       </c>
       <c r="P80" t="s">
-        <v>557</v>
+        <v>521</v>
       </c>
       <c r="Q80" t="s">
-        <v>423</v>
+        <v>522</v>
       </c>
       <c r="R80" t="s">
-        <v>558</v>
+        <v>523</v>
       </c>
       <c r="V80" t="s">
-        <v>425</v>
+        <v>322</v>
       </c>
     </row>
     <row r="81" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A81">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B81" t="s">
-        <v>559</v>
+        <v>524</v>
       </c>
       <c r="C81" t="s">
         <v>23</v>
       </c>
       <c r="H81" t="s">
-        <v>560</v>
+        <v>525</v>
       </c>
       <c r="K81" t="s">
-        <v>561</v>
+        <v>526</v>
       </c>
       <c r="M81" t="s">
-        <v>562</v>
+        <v>527</v>
       </c>
       <c r="N81" t="s">
         <v>27</v>
       </c>
       <c r="O81">
-        <v>61602</v>
+        <v>62298</v>
       </c>
       <c r="P81" t="s">
-        <v>562</v>
+        <v>528</v>
       </c>
       <c r="Q81" t="s">
-        <v>563</v>
+        <v>529</v>
       </c>
       <c r="R81" t="s">
-        <v>564</v>
+        <v>530</v>
       </c>
       <c r="V81" t="s">
-        <v>474</v>
+        <v>531</v>
       </c>
     </row>
     <row r="82" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A82">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B82" t="s">
-        <v>565</v>
+        <v>532</v>
       </c>
       <c r="C82" t="s">
         <v>23</v>
       </c>
       <c r="H82" t="s">
-        <v>566</v>
+        <v>533</v>
       </c>
       <c r="K82" t="s">
-        <v>567</v>
+        <v>534</v>
       </c>
       <c r="M82" t="s">
-        <v>568</v>
+        <v>535</v>
       </c>
       <c r="N82" t="s">
         <v>27</v>
       </c>
       <c r="O82">
-        <v>62274</v>
+        <v>62049</v>
       </c>
       <c r="P82" t="s">
-        <v>569</v>
-      </c>
-      <c r="Q82" s="2" t="s">
-        <v>769</v>
+        <v>536</v>
+      </c>
+      <c r="Q82" t="s">
+        <v>537</v>
       </c>
       <c r="R82" t="s">
-        <v>570</v>
+        <v>538</v>
       </c>
       <c r="V82" t="s">
-        <v>531</v>
+        <v>108</v>
       </c>
     </row>
     <row r="83" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A83">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B83" t="s">
-        <v>571</v>
+        <v>539</v>
       </c>
       <c r="C83" t="s">
         <v>23</v>
       </c>
       <c r="H83" t="s">
-        <v>572</v>
+        <v>540</v>
       </c>
       <c r="K83" t="s">
-        <v>573</v>
+        <v>541</v>
       </c>
       <c r="M83" t="s">
-        <v>574</v>
+        <v>542</v>
       </c>
       <c r="N83" t="s">
         <v>27</v>
       </c>
       <c r="O83">
-        <v>61856</v>
+        <v>62650</v>
       </c>
       <c r="P83" t="s">
-        <v>575</v>
+        <v>543</v>
       </c>
       <c r="Q83" t="s">
-        <v>576</v>
+        <v>544</v>
       </c>
       <c r="R83" t="s">
-        <v>577</v>
+        <v>545</v>
       </c>
       <c r="V83" t="s">
-        <v>100</v>
+        <v>283</v>
       </c>
     </row>
     <row r="84" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A84">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B84" t="s">
-        <v>578</v>
+        <v>546</v>
       </c>
       <c r="C84" t="s">
         <v>23</v>
       </c>
       <c r="H84" t="s">
-        <v>579</v>
+        <v>547</v>
       </c>
       <c r="K84" t="s">
-        <v>580</v>
+        <v>548</v>
       </c>
       <c r="M84" t="s">
-        <v>581</v>
+        <v>549</v>
       </c>
       <c r="N84" t="s">
         <v>27</v>
       </c>
       <c r="O84">
-        <v>62363</v>
+        <v>61951</v>
       </c>
       <c r="P84" t="s">
-        <v>582</v>
+        <v>550</v>
       </c>
       <c r="Q84" t="s">
-        <v>583</v>
+        <v>551</v>
       </c>
       <c r="R84" t="s">
-        <v>584</v>
+        <v>552</v>
       </c>
       <c r="V84" t="s">
-        <v>31</v>
+        <v>100</v>
       </c>
     </row>
     <row r="85" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A85">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B85" t="s">
-        <v>585</v>
+        <v>553</v>
       </c>
       <c r="C85" t="s">
         <v>23</v>
       </c>
       <c r="H85" t="s">
-        <v>586</v>
+        <v>554</v>
       </c>
       <c r="K85" t="s">
-        <v>587</v>
+        <v>555</v>
       </c>
       <c r="M85" t="s">
-        <v>588</v>
+        <v>556</v>
       </c>
       <c r="N85" t="s">
         <v>27</v>
       </c>
       <c r="O85">
-        <v>62938</v>
+        <v>61061</v>
       </c>
       <c r="P85" t="s">
-        <v>589</v>
+        <v>557</v>
       </c>
       <c r="Q85" t="s">
-        <v>37</v>
+        <v>423</v>
       </c>
       <c r="R85" t="s">
-        <v>590</v>
+        <v>558</v>
       </c>
       <c r="V85" t="s">
-        <v>39</v>
+        <v>425</v>
       </c>
     </row>
     <row r="86" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A86">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B86" t="s">
-        <v>591</v>
+        <v>559</v>
       </c>
       <c r="C86" t="s">
         <v>23</v>
       </c>
       <c r="H86" t="s">
-        <v>592</v>
+        <v>560</v>
       </c>
       <c r="K86" t="s">
-        <v>593</v>
+        <v>561</v>
       </c>
       <c r="M86" t="s">
-        <v>594</v>
+        <v>562</v>
       </c>
       <c r="N86" t="s">
         <v>27</v>
       </c>
       <c r="O86">
-        <v>62963</v>
+        <v>61602</v>
       </c>
       <c r="P86" t="s">
-        <v>595</v>
+        <v>562</v>
       </c>
       <c r="Q86" t="s">
-        <v>37</v>
+        <v>563</v>
       </c>
       <c r="R86" t="s">
-        <v>596</v>
+        <v>564</v>
       </c>
       <c r="V86" t="s">
-        <v>39</v>
+        <v>474</v>
       </c>
     </row>
     <row r="87" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A87">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B87" t="s">
-        <v>597</v>
+        <v>565</v>
       </c>
       <c r="C87" t="s">
         <v>23</v>
       </c>
       <c r="H87" t="s">
-        <v>598</v>
+        <v>566</v>
       </c>
       <c r="K87" t="s">
-        <v>599</v>
+        <v>567</v>
       </c>
       <c r="M87" t="s">
-        <v>600</v>
+        <v>568</v>
       </c>
       <c r="N87" t="s">
         <v>27</v>
       </c>
       <c r="O87">
-        <v>61327</v>
+        <v>62274</v>
       </c>
       <c r="P87" t="s">
-        <v>601</v>
-      </c>
-      <c r="Q87" t="s">
-        <v>602</v>
+        <v>569</v>
+      </c>
+      <c r="Q87" s="2" t="s">
+        <v>769</v>
       </c>
       <c r="R87" t="s">
-        <v>603</v>
+        <v>570</v>
       </c>
       <c r="V87" t="s">
-        <v>474</v>
+        <v>531</v>
       </c>
     </row>
     <row r="88" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A88">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B88" t="s">
-        <v>604</v>
+        <v>571</v>
       </c>
       <c r="C88" t="s">
         <v>23</v>
       </c>
       <c r="H88" t="s">
-        <v>605</v>
+        <v>572</v>
       </c>
       <c r="K88" t="s">
-        <v>606</v>
+        <v>573</v>
       </c>
       <c r="M88" t="s">
-        <v>607</v>
+        <v>574</v>
       </c>
       <c r="N88" t="s">
         <v>27</v>
       </c>
       <c r="O88">
-        <v>62233</v>
+        <v>61856</v>
       </c>
       <c r="P88" t="s">
-        <v>608</v>
+        <v>575</v>
       </c>
       <c r="Q88" t="s">
-        <v>609</v>
+        <v>576</v>
       </c>
       <c r="R88" t="s">
-        <v>610</v>
+        <v>577</v>
       </c>
       <c r="V88" t="s">
-        <v>531</v>
+        <v>100</v>
       </c>
     </row>
     <row r="89" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A89">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B89" t="s">
-        <v>611</v>
+        <v>578</v>
       </c>
       <c r="C89" t="s">
         <v>23</v>
       </c>
       <c r="H89" t="s">
-        <v>612</v>
+        <v>579</v>
       </c>
       <c r="K89" t="s">
-        <v>613</v>
+        <v>580</v>
       </c>
       <c r="M89" t="s">
-        <v>614</v>
+        <v>581</v>
       </c>
       <c r="N89" t="s">
         <v>27</v>
       </c>
       <c r="O89">
-        <v>62450</v>
+        <v>62363</v>
       </c>
       <c r="P89" t="s">
-        <v>615</v>
+        <v>582</v>
       </c>
       <c r="Q89" t="s">
-        <v>616</v>
+        <v>583</v>
       </c>
       <c r="R89" t="s">
-        <v>617</v>
+        <v>584</v>
       </c>
       <c r="V89" t="s">
-        <v>185</v>
+        <v>31</v>
       </c>
     </row>
     <row r="90" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A90">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B90" t="s">
-        <v>618</v>
+        <v>585</v>
       </c>
       <c r="C90" t="s">
         <v>23</v>
       </c>
       <c r="H90" t="s">
-        <v>619</v>
+        <v>586</v>
       </c>
       <c r="K90" t="s">
-        <v>620</v>
+        <v>587</v>
       </c>
       <c r="M90" t="s">
-        <v>621</v>
+        <v>588</v>
       </c>
       <c r="N90" t="s">
         <v>27</v>
       </c>
       <c r="O90">
-        <v>61201</v>
+        <v>62938</v>
       </c>
       <c r="P90" t="s">
-        <v>621</v>
+        <v>589</v>
       </c>
       <c r="Q90" t="s">
-        <v>622</v>
+        <v>37</v>
       </c>
       <c r="R90" t="s">
-        <v>623</v>
+        <v>590</v>
       </c>
       <c r="V90" t="s">
-        <v>322</v>
+        <v>39</v>
       </c>
     </row>
     <row r="91" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A91">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B91" t="s">
-        <v>624</v>
+        <v>591</v>
       </c>
       <c r="C91" t="s">
         <v>23</v>
       </c>
       <c r="H91" t="s">
-        <v>625</v>
+        <v>592</v>
       </c>
       <c r="K91" t="s">
-        <v>626</v>
+        <v>593</v>
       </c>
       <c r="M91" t="s">
-        <v>627</v>
+        <v>594</v>
       </c>
       <c r="N91" t="s">
         <v>27</v>
       </c>
       <c r="O91">
-        <v>62946</v>
+        <v>62963</v>
       </c>
       <c r="P91" t="s">
-        <v>628</v>
+        <v>595</v>
       </c>
       <c r="Q91" t="s">
         <v>37</v>
       </c>
       <c r="R91" t="s">
-        <v>629</v>
+        <v>596</v>
       </c>
       <c r="V91" t="s">
         <v>39</v>
@@ -6303,761 +6342,951 @@
     </row>
     <row r="92" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A92">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B92" t="s">
-        <v>630</v>
+        <v>597</v>
       </c>
       <c r="C92" t="s">
         <v>23</v>
       </c>
       <c r="H92" t="s">
-        <v>631</v>
+        <v>598</v>
       </c>
       <c r="K92" t="s">
-        <v>632</v>
+        <v>599</v>
       </c>
       <c r="M92" t="s">
-        <v>633</v>
+        <v>600</v>
       </c>
       <c r="N92" t="s">
         <v>27</v>
       </c>
       <c r="O92">
-        <v>62701</v>
+        <v>61327</v>
       </c>
       <c r="P92" t="s">
-        <v>634</v>
+        <v>601</v>
       </c>
       <c r="Q92" t="s">
-        <v>635</v>
+        <v>602</v>
       </c>
       <c r="R92" t="s">
-        <v>636</v>
+        <v>603</v>
       </c>
       <c r="V92" t="s">
-        <v>283</v>
+        <v>474</v>
       </c>
     </row>
     <row r="93" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A93">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="B93" t="s">
-        <v>637</v>
+        <v>604</v>
       </c>
       <c r="C93" t="s">
         <v>23</v>
       </c>
       <c r="H93" t="s">
-        <v>638</v>
+        <v>605</v>
       </c>
       <c r="K93" t="s">
-        <v>639</v>
+        <v>606</v>
       </c>
       <c r="M93" t="s">
-        <v>640</v>
+        <v>607</v>
       </c>
       <c r="N93" t="s">
         <v>27</v>
       </c>
       <c r="O93">
-        <v>62681</v>
+        <v>62233</v>
       </c>
       <c r="P93" t="s">
-        <v>641</v>
+        <v>608</v>
       </c>
       <c r="Q93" t="s">
-        <v>642</v>
+        <v>609</v>
       </c>
       <c r="R93" t="s">
-        <v>643</v>
+        <v>610</v>
       </c>
       <c r="V93" t="s">
-        <v>31</v>
+        <v>531</v>
       </c>
     </row>
     <row r="94" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A94">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B94" t="s">
-        <v>644</v>
+        <v>611</v>
       </c>
       <c r="C94" t="s">
         <v>23</v>
       </c>
       <c r="H94" t="s">
-        <v>645</v>
+        <v>612</v>
       </c>
       <c r="K94" t="s">
-        <v>646</v>
+        <v>613</v>
       </c>
       <c r="M94" t="s">
-        <v>647</v>
+        <v>614</v>
       </c>
       <c r="N94" t="s">
         <v>27</v>
       </c>
       <c r="O94">
-        <v>62694</v>
+        <v>62450</v>
       </c>
       <c r="P94" t="s">
-        <v>648</v>
-      </c>
-      <c r="Q94" s="2" t="s">
-        <v>765</v>
+        <v>615</v>
+      </c>
+      <c r="Q94" t="s">
+        <v>616</v>
       </c>
       <c r="R94" t="s">
-        <v>649</v>
+        <v>617</v>
       </c>
       <c r="V94" t="s">
-        <v>283</v>
+        <v>185</v>
       </c>
     </row>
     <row r="95" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A95">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B95" t="s">
-        <v>650</v>
+        <v>618</v>
       </c>
       <c r="C95" t="s">
         <v>23</v>
       </c>
       <c r="H95" t="s">
-        <v>651</v>
+        <v>619</v>
       </c>
       <c r="K95" t="s">
-        <v>652</v>
+        <v>620</v>
       </c>
       <c r="M95" t="s">
-        <v>653</v>
+        <v>621</v>
       </c>
       <c r="N95" t="s">
         <v>27</v>
       </c>
       <c r="O95">
-        <v>62565</v>
+        <v>61201</v>
       </c>
       <c r="P95" t="s">
-        <v>654</v>
+        <v>621</v>
       </c>
       <c r="Q95" t="s">
-        <v>768</v>
+        <v>622</v>
       </c>
       <c r="R95" t="s">
-        <v>655</v>
+        <v>623</v>
       </c>
       <c r="V95" t="s">
-        <v>108</v>
+        <v>322</v>
       </c>
     </row>
     <row r="96" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A96">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B96" t="s">
-        <v>656</v>
+        <v>624</v>
       </c>
       <c r="C96" t="s">
         <v>23</v>
       </c>
       <c r="H96" t="s">
-        <v>657</v>
+        <v>625</v>
       </c>
       <c r="K96" t="s">
-        <v>658</v>
+        <v>626</v>
       </c>
       <c r="M96" t="s">
-        <v>659</v>
+        <v>627</v>
       </c>
       <c r="N96" t="s">
         <v>27</v>
       </c>
       <c r="O96">
-        <v>62220</v>
+        <v>62946</v>
       </c>
       <c r="P96" t="s">
-        <v>660</v>
+        <v>628</v>
       </c>
       <c r="Q96" t="s">
-        <v>661</v>
+        <v>37</v>
       </c>
       <c r="R96" t="s">
-        <v>662</v>
+        <v>629</v>
       </c>
       <c r="V96" t="s">
-        <v>663</v>
+        <v>39</v>
       </c>
     </row>
     <row r="97" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A97">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B97" t="s">
-        <v>664</v>
+        <v>630</v>
       </c>
       <c r="C97" t="s">
         <v>23</v>
       </c>
       <c r="H97" t="s">
-        <v>665</v>
+        <v>631</v>
       </c>
       <c r="K97" t="s">
-        <v>666</v>
+        <v>632</v>
       </c>
       <c r="M97" t="s">
-        <v>667</v>
+        <v>633</v>
       </c>
       <c r="N97" t="s">
         <v>27</v>
       </c>
       <c r="O97">
-        <v>61483</v>
+        <v>62701</v>
       </c>
       <c r="P97" t="s">
-        <v>668</v>
+        <v>634</v>
       </c>
       <c r="Q97" t="s">
-        <v>669</v>
+        <v>635</v>
       </c>
       <c r="R97" t="s">
-        <v>670</v>
+        <v>636</v>
       </c>
       <c r="V97" t="s">
-        <v>474</v>
+        <v>283</v>
       </c>
     </row>
     <row r="98" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A98">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B98" t="s">
-        <v>671</v>
+        <v>637</v>
       </c>
       <c r="C98" t="s">
         <v>23</v>
       </c>
       <c r="H98" t="s">
-        <v>672</v>
+        <v>638</v>
       </c>
       <c r="K98" t="s">
-        <v>673</v>
+        <v>639</v>
       </c>
       <c r="M98" t="s">
-        <v>674</v>
+        <v>640</v>
       </c>
       <c r="N98" t="s">
         <v>27</v>
       </c>
       <c r="O98">
-        <v>61032</v>
+        <v>62681</v>
       </c>
       <c r="P98" t="s">
-        <v>675</v>
+        <v>641</v>
       </c>
       <c r="Q98" t="s">
-        <v>423</v>
+        <v>642</v>
       </c>
       <c r="R98" t="s">
-        <v>676</v>
+        <v>643</v>
       </c>
       <c r="V98" t="s">
-        <v>425</v>
+        <v>31</v>
       </c>
     </row>
     <row r="99" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A99">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B99" t="s">
-        <v>677</v>
+        <v>644</v>
       </c>
       <c r="C99" t="s">
         <v>23</v>
       </c>
       <c r="H99" t="s">
-        <v>678</v>
+        <v>645</v>
       </c>
       <c r="K99" t="s">
-        <v>679</v>
+        <v>646</v>
       </c>
       <c r="M99" t="s">
-        <v>680</v>
+        <v>647</v>
       </c>
       <c r="N99" t="s">
         <v>27</v>
       </c>
       <c r="O99">
-        <v>61554</v>
+        <v>62694</v>
       </c>
       <c r="P99" t="s">
-        <v>681</v>
-      </c>
-      <c r="Q99" t="s">
-        <v>682</v>
+        <v>648</v>
+      </c>
+      <c r="Q99" s="2" t="s">
+        <v>765</v>
       </c>
       <c r="R99" t="s">
-        <v>683</v>
+        <v>649</v>
       </c>
       <c r="V99" t="s">
-        <v>474</v>
+        <v>283</v>
       </c>
     </row>
     <row r="100" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A100">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B100" t="s">
-        <v>684</v>
+        <v>650</v>
       </c>
       <c r="C100" t="s">
         <v>23</v>
       </c>
       <c r="H100" t="s">
-        <v>685</v>
+        <v>651</v>
       </c>
       <c r="K100" t="s">
-        <v>686</v>
+        <v>652</v>
       </c>
       <c r="M100" t="s">
-        <v>687</v>
+        <v>653</v>
       </c>
       <c r="N100" t="s">
         <v>27</v>
       </c>
       <c r="O100">
-        <v>62952</v>
+        <v>62565</v>
       </c>
       <c r="P100" t="s">
-        <v>688</v>
+        <v>654</v>
       </c>
       <c r="Q100" t="s">
-        <v>689</v>
+        <v>768</v>
       </c>
       <c r="R100" t="s">
-        <v>690</v>
+        <v>655</v>
       </c>
       <c r="V100" t="s">
-        <v>39</v>
+        <v>108</v>
       </c>
     </row>
     <row r="101" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A101">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B101" t="s">
-        <v>691</v>
+        <v>656</v>
       </c>
       <c r="C101" t="s">
         <v>23</v>
       </c>
       <c r="H101" t="s">
-        <v>692</v>
+        <v>657</v>
       </c>
       <c r="K101" t="s">
-        <v>693</v>
+        <v>658</v>
       </c>
       <c r="M101" t="s">
-        <v>694</v>
+        <v>659</v>
       </c>
       <c r="N101" t="s">
         <v>27</v>
       </c>
       <c r="O101">
-        <v>61832</v>
+        <v>62220</v>
       </c>
       <c r="P101" t="s">
-        <v>695</v>
+        <v>660</v>
       </c>
       <c r="Q101" t="s">
-        <v>696</v>
+        <v>661</v>
       </c>
       <c r="R101" t="s">
-        <v>697</v>
+        <v>662</v>
       </c>
       <c r="V101" t="s">
-        <v>116</v>
+        <v>663</v>
       </c>
     </row>
     <row r="102" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A102">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B102" t="s">
-        <v>698</v>
+        <v>664</v>
       </c>
       <c r="C102" t="s">
         <v>23</v>
       </c>
       <c r="H102" t="s">
-        <v>699</v>
+        <v>665</v>
       </c>
       <c r="K102" t="s">
-        <v>700</v>
+        <v>666</v>
       </c>
       <c r="M102" t="s">
-        <v>701</v>
+        <v>667</v>
       </c>
       <c r="N102" t="s">
         <v>27</v>
       </c>
       <c r="O102">
-        <v>62863</v>
+        <v>61483</v>
       </c>
       <c r="P102" t="s">
-        <v>702</v>
+        <v>668</v>
       </c>
       <c r="Q102" t="s">
-        <v>183</v>
+        <v>669</v>
       </c>
       <c r="R102" t="s">
-        <v>703</v>
+        <v>670</v>
       </c>
       <c r="V102" t="s">
-        <v>185</v>
+        <v>474</v>
       </c>
     </row>
     <row r="103" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A103">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B103" t="s">
-        <v>704</v>
+        <v>671</v>
       </c>
       <c r="C103" t="s">
         <v>23</v>
       </c>
       <c r="H103" t="s">
-        <v>298</v>
+        <v>672</v>
       </c>
       <c r="K103" t="s">
-        <v>705</v>
+        <v>673</v>
       </c>
       <c r="M103" t="s">
-        <v>706</v>
+        <v>674</v>
       </c>
       <c r="N103" t="s">
         <v>27</v>
       </c>
       <c r="O103">
-        <v>61462</v>
+        <v>61032</v>
       </c>
       <c r="P103" t="s">
-        <v>707</v>
+        <v>675</v>
       </c>
       <c r="Q103" t="s">
-        <v>708</v>
+        <v>423</v>
       </c>
       <c r="R103" t="s">
-        <v>709</v>
+        <v>676</v>
       </c>
       <c r="V103" t="s">
-        <v>270</v>
+        <v>425</v>
       </c>
     </row>
     <row r="104" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A104">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B104" t="s">
-        <v>710</v>
+        <v>677</v>
       </c>
       <c r="C104" t="s">
         <v>23</v>
       </c>
       <c r="H104" t="s">
-        <v>711</v>
+        <v>678</v>
       </c>
       <c r="K104" t="s">
-        <v>712</v>
+        <v>679</v>
       </c>
       <c r="M104" t="s">
-        <v>713</v>
+        <v>680</v>
       </c>
       <c r="N104" t="s">
         <v>27</v>
       </c>
       <c r="O104">
-        <v>62263</v>
+        <v>61554</v>
       </c>
       <c r="P104" t="s">
-        <v>714</v>
+        <v>681</v>
       </c>
       <c r="Q104" t="s">
-        <v>715</v>
+        <v>682</v>
       </c>
       <c r="R104" t="s">
-        <v>716</v>
+        <v>683</v>
       </c>
       <c r="V104" t="s">
-        <v>531</v>
+        <v>474</v>
       </c>
     </row>
     <row r="105" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A105">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B105" t="s">
-        <v>717</v>
+        <v>684</v>
       </c>
       <c r="C105" t="s">
         <v>23</v>
       </c>
       <c r="H105" t="s">
-        <v>718</v>
+        <v>685</v>
       </c>
       <c r="K105" t="s">
-        <v>719</v>
+        <v>686</v>
       </c>
       <c r="M105" t="s">
-        <v>720</v>
+        <v>687</v>
       </c>
       <c r="N105" t="s">
         <v>27</v>
       </c>
       <c r="O105">
-        <v>62837</v>
+        <v>62952</v>
       </c>
       <c r="P105" t="s">
-        <v>721</v>
+        <v>688</v>
       </c>
       <c r="Q105" t="s">
-        <v>722</v>
+        <v>689</v>
       </c>
       <c r="R105" t="s">
-        <v>723</v>
+        <v>690</v>
       </c>
       <c r="V105" t="s">
-        <v>185</v>
+        <v>39</v>
       </c>
     </row>
     <row r="106" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A106">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B106" t="s">
-        <v>724</v>
+        <v>691</v>
       </c>
       <c r="C106" t="s">
         <v>23</v>
       </c>
       <c r="H106" t="s">
-        <v>725</v>
+        <v>692</v>
       </c>
       <c r="K106" t="s">
-        <v>726</v>
+        <v>693</v>
       </c>
       <c r="M106" t="s">
-        <v>727</v>
+        <v>694</v>
       </c>
       <c r="N106" t="s">
         <v>27</v>
       </c>
       <c r="O106">
-        <v>62821</v>
+        <v>61832</v>
       </c>
       <c r="P106" t="s">
-        <v>728</v>
+        <v>695</v>
       </c>
       <c r="Q106" t="s">
-        <v>183</v>
+        <v>696</v>
       </c>
       <c r="R106" t="s">
-        <v>729</v>
+        <v>697</v>
       </c>
       <c r="V106" t="s">
-        <v>185</v>
+        <v>116</v>
       </c>
     </row>
     <row r="107" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A107">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B107" t="s">
-        <v>730</v>
+        <v>698</v>
       </c>
       <c r="C107" t="s">
         <v>23</v>
       </c>
       <c r="H107" t="s">
-        <v>731</v>
+        <v>699</v>
       </c>
       <c r="K107" t="s">
-        <v>732</v>
+        <v>700</v>
       </c>
       <c r="M107" t="s">
-        <v>733</v>
+        <v>701</v>
       </c>
       <c r="N107" t="s">
         <v>27</v>
       </c>
       <c r="O107">
-        <v>61270</v>
+        <v>62863</v>
       </c>
       <c r="P107" t="s">
-        <v>734</v>
+        <v>702</v>
       </c>
       <c r="Q107" t="s">
-        <v>735</v>
+        <v>183</v>
       </c>
       <c r="R107" t="s">
-        <v>736</v>
+        <v>703</v>
       </c>
       <c r="V107" t="s">
-        <v>322</v>
+        <v>185</v>
       </c>
     </row>
     <row r="108" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A108">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B108" t="s">
-        <v>737</v>
+        <v>704</v>
       </c>
       <c r="C108" t="s">
         <v>23</v>
       </c>
       <c r="H108" t="s">
-        <v>738</v>
+        <v>298</v>
       </c>
       <c r="K108" t="s">
-        <v>739</v>
+        <v>705</v>
       </c>
       <c r="M108" t="s">
-        <v>740</v>
+        <v>706</v>
       </c>
       <c r="N108" t="s">
         <v>27</v>
       </c>
       <c r="O108">
-        <v>60432</v>
+        <v>61462</v>
       </c>
       <c r="P108" t="s">
-        <v>741</v>
+        <v>707</v>
       </c>
       <c r="Q108" t="s">
-        <v>742</v>
+        <v>708</v>
       </c>
       <c r="R108" t="s">
-        <v>743</v>
+        <v>709</v>
       </c>
       <c r="V108" t="s">
-        <v>744</v>
+        <v>270</v>
       </c>
     </row>
     <row r="109" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A109">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B109" t="s">
-        <v>745</v>
+        <v>710</v>
       </c>
       <c r="C109" t="s">
         <v>23</v>
       </c>
       <c r="H109" t="s">
-        <v>746</v>
+        <v>711</v>
       </c>
       <c r="K109" t="s">
-        <v>747</v>
+        <v>712</v>
       </c>
       <c r="M109" t="s">
-        <v>465</v>
+        <v>713</v>
       </c>
       <c r="N109" t="s">
         <v>27</v>
       </c>
       <c r="O109">
-        <v>62959</v>
+        <v>62263</v>
       </c>
       <c r="P109" t="s">
-        <v>748</v>
+        <v>714</v>
       </c>
       <c r="Q109" t="s">
-        <v>37</v>
+        <v>715</v>
       </c>
       <c r="R109" t="s">
-        <v>749</v>
+        <v>716</v>
       </c>
       <c r="V109" t="s">
-        <v>39</v>
+        <v>531</v>
       </c>
     </row>
     <row r="110" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A110">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B110" t="s">
-        <v>750</v>
+        <v>717</v>
       </c>
       <c r="C110" t="s">
         <v>23</v>
       </c>
       <c r="H110" t="s">
-        <v>751</v>
+        <v>718</v>
       </c>
       <c r="K110" t="s">
-        <v>752</v>
+        <v>719</v>
       </c>
       <c r="M110" t="s">
-        <v>753</v>
+        <v>720</v>
       </c>
       <c r="N110" t="s">
         <v>27</v>
       </c>
       <c r="O110">
-        <v>61101</v>
+        <v>62837</v>
       </c>
       <c r="P110" t="s">
-        <v>754</v>
+        <v>721</v>
       </c>
       <c r="Q110" t="s">
-        <v>755</v>
+        <v>722</v>
       </c>
       <c r="R110" t="s">
-        <v>756</v>
+        <v>723</v>
       </c>
       <c r="V110" t="s">
-        <v>55</v>
+        <v>185</v>
       </c>
     </row>
     <row r="111" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A111">
+        <v>97</v>
+      </c>
+      <c r="B111" t="s">
+        <v>724</v>
+      </c>
+      <c r="C111" t="s">
+        <v>23</v>
+      </c>
+      <c r="H111" t="s">
+        <v>725</v>
+      </c>
+      <c r="K111" t="s">
+        <v>726</v>
+      </c>
+      <c r="M111" t="s">
+        <v>727</v>
+      </c>
+      <c r="N111" t="s">
+        <v>27</v>
+      </c>
+      <c r="O111">
+        <v>62821</v>
+      </c>
+      <c r="P111" t="s">
+        <v>728</v>
+      </c>
+      <c r="Q111" t="s">
+        <v>183</v>
+      </c>
+      <c r="R111" t="s">
+        <v>729</v>
+      </c>
+      <c r="V111" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="112" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A112">
+        <v>98</v>
+      </c>
+      <c r="B112" t="s">
+        <v>730</v>
+      </c>
+      <c r="C112" t="s">
+        <v>23</v>
+      </c>
+      <c r="H112" t="s">
+        <v>731</v>
+      </c>
+      <c r="K112" t="s">
+        <v>732</v>
+      </c>
+      <c r="M112" t="s">
+        <v>733</v>
+      </c>
+      <c r="N112" t="s">
+        <v>27</v>
+      </c>
+      <c r="O112">
+        <v>61270</v>
+      </c>
+      <c r="P112" t="s">
+        <v>734</v>
+      </c>
+      <c r="Q112" t="s">
+        <v>735</v>
+      </c>
+      <c r="R112" t="s">
+        <v>736</v>
+      </c>
+      <c r="V112" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="113" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A113">
+        <v>99</v>
+      </c>
+      <c r="B113" t="s">
+        <v>737</v>
+      </c>
+      <c r="C113" t="s">
+        <v>23</v>
+      </c>
+      <c r="H113" t="s">
+        <v>738</v>
+      </c>
+      <c r="K113" t="s">
+        <v>739</v>
+      </c>
+      <c r="M113" t="s">
+        <v>740</v>
+      </c>
+      <c r="N113" t="s">
+        <v>27</v>
+      </c>
+      <c r="O113">
+        <v>60432</v>
+      </c>
+      <c r="P113" t="s">
+        <v>741</v>
+      </c>
+      <c r="Q113" t="s">
+        <v>742</v>
+      </c>
+      <c r="R113" t="s">
+        <v>743</v>
+      </c>
+      <c r="V113" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="114" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A114">
+        <v>100</v>
+      </c>
+      <c r="B114" t="s">
+        <v>745</v>
+      </c>
+      <c r="C114" t="s">
+        <v>23</v>
+      </c>
+      <c r="H114" t="s">
+        <v>746</v>
+      </c>
+      <c r="K114" t="s">
+        <v>747</v>
+      </c>
+      <c r="M114" t="s">
+        <v>465</v>
+      </c>
+      <c r="N114" t="s">
+        <v>27</v>
+      </c>
+      <c r="O114">
+        <v>62959</v>
+      </c>
+      <c r="P114" t="s">
+        <v>748</v>
+      </c>
+      <c r="Q114" t="s">
+        <v>37</v>
+      </c>
+      <c r="R114" t="s">
+        <v>749</v>
+      </c>
+      <c r="V114" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="115" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A115">
+        <v>101</v>
+      </c>
+      <c r="B115" t="s">
+        <v>750</v>
+      </c>
+      <c r="C115" t="s">
+        <v>23</v>
+      </c>
+      <c r="H115" t="s">
+        <v>751</v>
+      </c>
+      <c r="K115" t="s">
+        <v>752</v>
+      </c>
+      <c r="M115" t="s">
+        <v>753</v>
+      </c>
+      <c r="N115" t="s">
+        <v>27</v>
+      </c>
+      <c r="O115">
+        <v>61101</v>
+      </c>
+      <c r="P115" t="s">
+        <v>754</v>
+      </c>
+      <c r="Q115" t="s">
+        <v>755</v>
+      </c>
+      <c r="R115" t="s">
+        <v>756</v>
+      </c>
+      <c r="V115" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="116" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A116">
         <v>102</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B116" t="s">
         <v>757</v>
       </c>
-      <c r="C111" t="s">
-        <v>23</v>
-      </c>
-      <c r="H111" t="s">
+      <c r="C116" t="s">
+        <v>23</v>
+      </c>
+      <c r="H116" t="s">
         <v>758</v>
       </c>
-      <c r="K111" t="s">
+      <c r="K116" t="s">
         <v>759</v>
       </c>
-      <c r="M111" t="s">
+      <c r="M116" t="s">
         <v>760</v>
       </c>
-      <c r="N111" t="s">
-        <v>27</v>
-      </c>
-      <c r="O111">
+      <c r="N116" t="s">
+        <v>27</v>
+      </c>
+      <c r="O116">
         <v>61530</v>
       </c>
-      <c r="P111" t="s">
+      <c r="P116" t="s">
         <v>761</v>
       </c>
-      <c r="Q111" t="s">
+      <c r="Q116" t="s">
         <v>762</v>
       </c>
-      <c r="R111" t="s">
+      <c r="R116" t="s">
         <v>763</v>
       </c>
-      <c r="V111" t="s">
+      <c r="V116" t="s">
         <v>255</v>
       </c>
     </row>
@@ -7068,9 +7297,9 @@
     <hyperlink ref="Q45" r:id="rId3" xr:uid="{E8701583-F1BF-4A71-A500-C737411446E5}"/>
     <hyperlink ref="Q44" r:id="rId4" xr:uid="{9BB64827-CBE0-4F72-88A8-10DFB32413E9}"/>
     <hyperlink ref="Q49" r:id="rId5" xr:uid="{231A7501-BA49-418B-817D-98BB18CD74C8}"/>
-    <hyperlink ref="Q60" r:id="rId6" xr:uid="{4B7E1D46-47BF-4923-887D-F0D311096F3B}"/>
-    <hyperlink ref="Q82" r:id="rId7" xr:uid="{968EC501-FFBE-489E-849D-C2279F57E36E}"/>
-    <hyperlink ref="Q94" r:id="rId8" xr:uid="{EDF05CEF-DF2C-4746-B08F-B2D45EF1CA5F}"/>
+    <hyperlink ref="Q65" r:id="rId6" xr:uid="{4B7E1D46-47BF-4923-887D-F0D311096F3B}"/>
+    <hyperlink ref="Q87" r:id="rId7" xr:uid="{968EC501-FFBE-489E-849D-C2279F57E36E}"/>
+    <hyperlink ref="Q99" r:id="rId8" xr:uid="{EDF05CEF-DF2C-4746-B08F-B2D45EF1CA5F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
added il_courts_plus.xlsx as interim list during transition
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/il_courts.xlsx
+++ b/docassemble/ILAO/data/sources/il_courts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\local-DA-easyforms-dev\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3866A7E-5F96-4F20-9E44-E29745CE2B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF8AA1E2-2857-4B60-B135-6803DF63A830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28995" yWindow="-3000" windowWidth="27120" windowHeight="17865" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1163" uniqueCount="783">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="770">
   <si>
     <t>court_code</t>
   </si>
@@ -2335,45 +2335,6 @@
   </si>
   <si>
     <t>https://24thcircuit.illinoiscourts.gov/</t>
-  </si>
-  <si>
-    <t>Kane County Judicial Center</t>
-  </si>
-  <si>
-    <t>37W777 Route 38</t>
-  </si>
-  <si>
-    <t>St. Charles</t>
-  </si>
-  <si>
-    <t>Kane County Juvenile Justice Center</t>
-  </si>
-  <si>
-    <t>37W655 Route 38</t>
-  </si>
-  <si>
-    <t>530 S. Randall Road</t>
-  </si>
-  <si>
-    <t>Aurora Branch Court</t>
-  </si>
-  <si>
-    <t>1200 East Indian Trail Road</t>
-  </si>
-  <si>
-    <t>Aurora</t>
-  </si>
-  <si>
-    <t>Elgin</t>
-  </si>
-  <si>
-    <t>Elgin Branch Court</t>
-  </si>
-  <si>
-    <t>150 Dexter Court</t>
-  </si>
-  <si>
-    <t>Kane County Branch Court</t>
   </si>
 </sst>
 </file>
@@ -2825,7 +2786,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V116"/>
+  <dimension ref="A1:V111"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" customWidth="1"/>
@@ -4936,759 +4897,759 @@
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>111</v>
+        <v>46</v>
       </c>
       <c r="B55" t="s">
-        <v>770</v>
+        <v>377</v>
       </c>
       <c r="C55" t="s">
         <v>23</v>
       </c>
       <c r="H55" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="K55" t="s">
-        <v>771</v>
+        <v>379</v>
       </c>
       <c r="M55" t="s">
-        <v>772</v>
+        <v>380</v>
       </c>
       <c r="N55" t="s">
         <v>27</v>
       </c>
       <c r="O55">
-        <v>60175</v>
+        <v>60901</v>
       </c>
       <c r="P55" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="Q55" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="R55" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="V55" t="s">
-        <v>376</v>
+        <v>330</v>
       </c>
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>112</v>
+        <v>47</v>
       </c>
       <c r="B56" t="s">
-        <v>773</v>
+        <v>383</v>
       </c>
       <c r="C56" t="s">
         <v>23</v>
       </c>
       <c r="H56" t="s">
-        <v>370</v>
+        <v>384</v>
       </c>
       <c r="K56" t="s">
-        <v>774</v>
+        <v>385</v>
       </c>
       <c r="M56" t="s">
-        <v>772</v>
+        <v>386</v>
       </c>
       <c r="N56" t="s">
         <v>27</v>
       </c>
       <c r="O56">
-        <v>60174</v>
+        <v>60560</v>
       </c>
       <c r="P56" t="s">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="Q56" t="s">
-        <v>374</v>
+        <v>388</v>
       </c>
       <c r="R56" t="s">
-        <v>375</v>
+        <v>389</v>
       </c>
       <c r="V56" t="s">
-        <v>376</v>
+        <v>200</v>
       </c>
     </row>
     <row r="57" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>113</v>
+        <v>48</v>
       </c>
       <c r="B57" t="s">
-        <v>782</v>
+        <v>390</v>
       </c>
       <c r="C57" t="s">
         <v>23</v>
       </c>
       <c r="H57" t="s">
-        <v>370</v>
+        <v>391</v>
       </c>
       <c r="K57" t="s">
-        <v>775</v>
+        <v>392</v>
       </c>
       <c r="M57" t="s">
-        <v>772</v>
+        <v>393</v>
       </c>
       <c r="N57" t="s">
         <v>27</v>
       </c>
       <c r="O57">
-        <v>60174</v>
+        <v>61401</v>
       </c>
       <c r="P57" t="s">
-        <v>373</v>
+        <v>394</v>
       </c>
       <c r="Q57" t="s">
-        <v>374</v>
+        <v>395</v>
       </c>
       <c r="R57" t="s">
-        <v>375</v>
+        <v>396</v>
       </c>
       <c r="V57" t="s">
-        <v>376</v>
+        <v>270</v>
       </c>
     </row>
     <row r="58" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A58">
-        <v>114</v>
+        <v>49</v>
       </c>
       <c r="B58" t="s">
-        <v>776</v>
+        <v>397</v>
       </c>
       <c r="C58" t="s">
         <v>23</v>
       </c>
       <c r="H58" t="s">
-        <v>370</v>
+        <v>398</v>
       </c>
       <c r="K58" t="s">
-        <v>777</v>
+        <v>399</v>
       </c>
       <c r="M58" t="s">
-        <v>778</v>
+        <v>400</v>
       </c>
       <c r="N58" t="s">
         <v>27</v>
       </c>
       <c r="O58">
-        <v>60505</v>
+        <v>60085</v>
       </c>
       <c r="P58" t="s">
-        <v>373</v>
+        <v>401</v>
       </c>
       <c r="Q58" t="s">
-        <v>374</v>
+        <v>402</v>
       </c>
       <c r="R58" t="s">
-        <v>375</v>
+        <v>403</v>
       </c>
       <c r="V58" t="s">
-        <v>376</v>
+        <v>404</v>
       </c>
     </row>
     <row r="59" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="B59" t="s">
-        <v>780</v>
+        <v>405</v>
       </c>
       <c r="C59" t="s">
         <v>23</v>
       </c>
       <c r="H59" t="s">
-        <v>370</v>
+        <v>406</v>
       </c>
       <c r="K59" t="s">
-        <v>781</v>
+        <v>407</v>
       </c>
       <c r="M59" t="s">
-        <v>779</v>
+        <v>408</v>
       </c>
       <c r="N59" t="s">
         <v>27</v>
       </c>
       <c r="O59">
-        <v>60120</v>
+        <v>61350</v>
       </c>
       <c r="P59" t="s">
-        <v>373</v>
+        <v>409</v>
       </c>
       <c r="Q59" t="s">
-        <v>374</v>
+        <v>410</v>
       </c>
       <c r="R59" t="s">
-        <v>375</v>
+        <v>411</v>
       </c>
       <c r="V59" t="s">
-        <v>376</v>
+        <v>70</v>
       </c>
     </row>
     <row r="60" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B60" t="s">
-        <v>377</v>
+        <v>412</v>
       </c>
       <c r="C60" t="s">
         <v>23</v>
       </c>
       <c r="H60" t="s">
-        <v>378</v>
+        <v>413</v>
       </c>
       <c r="K60" t="s">
-        <v>379</v>
+        <v>414</v>
       </c>
       <c r="M60" t="s">
-        <v>380</v>
+        <v>415</v>
       </c>
       <c r="N60" t="s">
         <v>27</v>
       </c>
       <c r="O60">
-        <v>60901</v>
+        <v>62439</v>
       </c>
       <c r="P60" t="s">
-        <v>380</v>
-      </c>
-      <c r="Q60" t="s">
-        <v>381</v>
+        <v>416</v>
+      </c>
+      <c r="Q60" s="2" t="s">
+        <v>767</v>
       </c>
       <c r="R60" t="s">
-        <v>382</v>
+        <v>417</v>
       </c>
       <c r="V60" t="s">
-        <v>330</v>
+        <v>185</v>
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B61" t="s">
-        <v>383</v>
+        <v>418</v>
       </c>
       <c r="C61" t="s">
         <v>23</v>
       </c>
       <c r="H61" t="s">
-        <v>384</v>
+        <v>419</v>
       </c>
       <c r="K61" t="s">
-        <v>385</v>
+        <v>420</v>
       </c>
       <c r="M61" t="s">
-        <v>386</v>
+        <v>421</v>
       </c>
       <c r="N61" t="s">
         <v>27</v>
       </c>
       <c r="O61">
-        <v>60560</v>
+        <v>61021</v>
       </c>
       <c r="P61" t="s">
-        <v>387</v>
+        <v>422</v>
       </c>
       <c r="Q61" t="s">
-        <v>388</v>
+        <v>423</v>
       </c>
       <c r="R61" t="s">
-        <v>389</v>
+        <v>424</v>
       </c>
       <c r="V61" t="s">
-        <v>200</v>
+        <v>425</v>
       </c>
     </row>
     <row r="62" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B62" t="s">
-        <v>390</v>
+        <v>426</v>
       </c>
       <c r="C62" t="s">
         <v>23</v>
       </c>
       <c r="H62" t="s">
-        <v>391</v>
+        <v>427</v>
       </c>
       <c r="K62" t="s">
-        <v>392</v>
+        <v>428</v>
       </c>
       <c r="M62" t="s">
-        <v>393</v>
+        <v>429</v>
       </c>
       <c r="N62" t="s">
         <v>27</v>
       </c>
       <c r="O62">
-        <v>61401</v>
+        <v>61764</v>
       </c>
       <c r="P62" t="s">
-        <v>394</v>
+        <v>430</v>
       </c>
       <c r="Q62" t="s">
-        <v>395</v>
+        <v>431</v>
       </c>
       <c r="R62" t="s">
-        <v>396</v>
+        <v>432</v>
       </c>
       <c r="V62" t="s">
-        <v>270</v>
+        <v>255</v>
       </c>
     </row>
     <row r="63" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B63" t="s">
-        <v>397</v>
+        <v>433</v>
       </c>
       <c r="C63" t="s">
         <v>23</v>
       </c>
       <c r="H63" t="s">
-        <v>398</v>
+        <v>434</v>
       </c>
       <c r="K63" t="s">
-        <v>399</v>
+        <v>435</v>
       </c>
       <c r="M63" t="s">
-        <v>400</v>
+        <v>436</v>
       </c>
       <c r="N63" t="s">
         <v>27</v>
       </c>
       <c r="O63">
-        <v>60085</v>
+        <v>62656</v>
       </c>
       <c r="P63" t="s">
-        <v>401</v>
+        <v>437</v>
       </c>
       <c r="Q63" t="s">
-        <v>402</v>
+        <v>438</v>
       </c>
       <c r="R63" t="s">
-        <v>403</v>
+        <v>439</v>
       </c>
       <c r="V63" t="s">
-        <v>404</v>
+        <v>255</v>
       </c>
     </row>
     <row r="64" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A64">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B64" t="s">
-        <v>405</v>
+        <v>440</v>
       </c>
       <c r="C64" t="s">
         <v>23</v>
       </c>
       <c r="H64" t="s">
-        <v>406</v>
+        <v>441</v>
       </c>
       <c r="K64" t="s">
-        <v>407</v>
+        <v>442</v>
       </c>
       <c r="M64" t="s">
-        <v>408</v>
+        <v>443</v>
       </c>
       <c r="N64" t="s">
         <v>27</v>
       </c>
       <c r="O64">
-        <v>61350</v>
+        <v>62523</v>
       </c>
       <c r="P64" t="s">
-        <v>409</v>
+        <v>444</v>
       </c>
       <c r="Q64" t="s">
-        <v>410</v>
+        <v>445</v>
       </c>
       <c r="R64" t="s">
-        <v>411</v>
+        <v>446</v>
       </c>
       <c r="V64" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="65" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B65" t="s">
-        <v>412</v>
+        <v>447</v>
       </c>
       <c r="C65" t="s">
         <v>23</v>
       </c>
       <c r="H65" t="s">
-        <v>413</v>
+        <v>448</v>
       </c>
       <c r="K65" t="s">
-        <v>414</v>
+        <v>449</v>
       </c>
       <c r="M65" t="s">
-        <v>415</v>
+        <v>450</v>
       </c>
       <c r="N65" t="s">
         <v>27</v>
       </c>
       <c r="O65">
-        <v>62439</v>
+        <v>62626</v>
       </c>
       <c r="P65" t="s">
-        <v>416</v>
-      </c>
-      <c r="Q65" s="2" t="s">
-        <v>767</v>
+        <v>451</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>452</v>
       </c>
       <c r="R65" t="s">
-        <v>417</v>
+        <v>453</v>
       </c>
       <c r="V65" t="s">
-        <v>185</v>
+        <v>283</v>
       </c>
     </row>
     <row r="66" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B66" t="s">
-        <v>418</v>
+        <v>454</v>
       </c>
       <c r="C66" t="s">
         <v>23</v>
       </c>
       <c r="H66" t="s">
-        <v>419</v>
+        <v>455</v>
       </c>
       <c r="K66" t="s">
-        <v>420</v>
+        <v>456</v>
       </c>
       <c r="M66" t="s">
-        <v>421</v>
+        <v>457</v>
       </c>
       <c r="N66" t="s">
         <v>27</v>
       </c>
       <c r="O66">
-        <v>61021</v>
+        <v>62025</v>
       </c>
       <c r="P66" t="s">
-        <v>422</v>
+        <v>458</v>
       </c>
       <c r="Q66" t="s">
-        <v>423</v>
+        <v>459</v>
       </c>
       <c r="R66" t="s">
-        <v>424</v>
+        <v>460</v>
       </c>
       <c r="V66" t="s">
-        <v>425</v>
+        <v>47</v>
       </c>
     </row>
     <row r="67" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B67" t="s">
-        <v>426</v>
+        <v>461</v>
       </c>
       <c r="C67" t="s">
         <v>23</v>
       </c>
       <c r="H67" t="s">
-        <v>427</v>
+        <v>462</v>
       </c>
       <c r="K67" t="s">
-        <v>428</v>
+        <v>463</v>
       </c>
       <c r="M67" t="s">
-        <v>429</v>
+        <v>464</v>
       </c>
       <c r="N67" t="s">
         <v>27</v>
       </c>
       <c r="O67">
-        <v>61764</v>
+        <v>62881</v>
       </c>
       <c r="P67" t="s">
-        <v>430</v>
+        <v>465</v>
       </c>
       <c r="Q67" t="s">
-        <v>431</v>
+        <v>466</v>
       </c>
       <c r="R67" t="s">
-        <v>432</v>
+        <v>467</v>
       </c>
       <c r="V67" t="s">
-        <v>255</v>
+        <v>108</v>
       </c>
     </row>
     <row r="68" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B68" t="s">
-        <v>433</v>
+        <v>468</v>
       </c>
       <c r="C68" t="s">
         <v>23</v>
       </c>
       <c r="H68" t="s">
-        <v>434</v>
+        <v>469</v>
       </c>
       <c r="K68" t="s">
-        <v>435</v>
+        <v>470</v>
       </c>
       <c r="M68" t="s">
-        <v>436</v>
+        <v>471</v>
       </c>
       <c r="N68" t="s">
         <v>27</v>
       </c>
       <c r="O68">
-        <v>62656</v>
+        <v>61540</v>
       </c>
       <c r="P68" t="s">
-        <v>437</v>
+        <v>112</v>
       </c>
       <c r="Q68" t="s">
-        <v>438</v>
+        <v>472</v>
       </c>
       <c r="R68" t="s">
-        <v>439</v>
+        <v>473</v>
       </c>
       <c r="V68" t="s">
-        <v>255</v>
+        <v>474</v>
       </c>
     </row>
     <row r="69" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A69">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B69" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="C69" t="s">
         <v>23</v>
       </c>
       <c r="H69" t="s">
-        <v>441</v>
+        <v>476</v>
       </c>
       <c r="K69" t="s">
-        <v>442</v>
+        <v>477</v>
       </c>
       <c r="M69" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="N69" t="s">
         <v>27</v>
       </c>
       <c r="O69">
-        <v>62523</v>
+        <v>62644</v>
       </c>
       <c r="P69" t="s">
-        <v>444</v>
+        <v>479</v>
       </c>
       <c r="Q69" t="s">
-        <v>445</v>
+        <v>480</v>
       </c>
       <c r="R69" t="s">
-        <v>446</v>
+        <v>481</v>
       </c>
       <c r="V69" t="s">
-        <v>100</v>
+        <v>31</v>
       </c>
     </row>
     <row r="70" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A70">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B70" t="s">
-        <v>447</v>
+        <v>482</v>
       </c>
       <c r="C70" t="s">
         <v>23</v>
       </c>
       <c r="H70" t="s">
-        <v>448</v>
+        <v>483</v>
       </c>
       <c r="K70" t="s">
-        <v>449</v>
+        <v>484</v>
       </c>
       <c r="M70" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="N70" t="s">
         <v>27</v>
       </c>
       <c r="O70">
-        <v>62626</v>
+        <v>62960</v>
       </c>
       <c r="P70" t="s">
-        <v>451</v>
+        <v>486</v>
       </c>
       <c r="Q70" t="s">
-        <v>452</v>
+        <v>37</v>
       </c>
       <c r="R70" t="s">
-        <v>453</v>
+        <v>487</v>
       </c>
       <c r="V70" t="s">
-        <v>283</v>
+        <v>39</v>
       </c>
     </row>
     <row r="71" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A71">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B71" t="s">
-        <v>454</v>
+        <v>488</v>
       </c>
       <c r="C71" t="s">
         <v>23</v>
       </c>
       <c r="H71" t="s">
-        <v>455</v>
+        <v>489</v>
       </c>
       <c r="K71" t="s">
-        <v>456</v>
+        <v>490</v>
       </c>
       <c r="M71" t="s">
-        <v>457</v>
+        <v>491</v>
       </c>
       <c r="N71" t="s">
         <v>27</v>
       </c>
       <c r="O71">
-        <v>62025</v>
+        <v>61455</v>
       </c>
       <c r="P71" t="s">
-        <v>458</v>
+        <v>492</v>
       </c>
       <c r="Q71" t="s">
-        <v>459</v>
+        <v>493</v>
       </c>
       <c r="R71" t="s">
-        <v>460</v>
+        <v>494</v>
       </c>
       <c r="V71" t="s">
-        <v>47</v>
+        <v>270</v>
       </c>
     </row>
     <row r="72" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A72">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B72" t="s">
-        <v>461</v>
+        <v>495</v>
       </c>
       <c r="C72" t="s">
         <v>23</v>
       </c>
       <c r="H72" t="s">
-        <v>462</v>
+        <v>496</v>
       </c>
       <c r="K72" t="s">
-        <v>463</v>
+        <v>497</v>
       </c>
       <c r="M72" t="s">
-        <v>464</v>
+        <v>498</v>
       </c>
       <c r="N72" t="s">
         <v>27</v>
       </c>
       <c r="O72">
-        <v>62881</v>
+        <v>60098</v>
       </c>
       <c r="P72" t="s">
-        <v>465</v>
+        <v>499</v>
       </c>
       <c r="Q72" t="s">
-        <v>466</v>
+        <v>500</v>
       </c>
       <c r="R72" t="s">
-        <v>467</v>
+        <v>501</v>
       </c>
       <c r="V72" t="s">
-        <v>108</v>
+        <v>502</v>
       </c>
     </row>
     <row r="73" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A73">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B73" t="s">
-        <v>468</v>
+        <v>503</v>
       </c>
       <c r="C73" t="s">
         <v>23</v>
       </c>
       <c r="H73" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
       <c r="K73" t="s">
-        <v>470</v>
+        <v>505</v>
       </c>
       <c r="M73" t="s">
-        <v>471</v>
+        <v>506</v>
       </c>
       <c r="N73" t="s">
         <v>27</v>
       </c>
       <c r="O73">
-        <v>61540</v>
+        <v>61701</v>
       </c>
       <c r="P73" t="s">
-        <v>112</v>
+        <v>507</v>
       </c>
       <c r="Q73" t="s">
-        <v>472</v>
+        <v>508</v>
       </c>
       <c r="R73" t="s">
-        <v>473</v>
+        <v>509</v>
       </c>
       <c r="V73" t="s">
-        <v>474</v>
+        <v>255</v>
       </c>
     </row>
     <row r="74" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A74">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B74" t="s">
-        <v>475</v>
+        <v>510</v>
       </c>
       <c r="C74" t="s">
         <v>23</v>
       </c>
       <c r="H74" t="s">
-        <v>476</v>
+        <v>511</v>
       </c>
       <c r="K74" t="s">
-        <v>477</v>
+        <v>512</v>
       </c>
       <c r="M74" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
       <c r="N74" t="s">
         <v>27</v>
       </c>
       <c r="O74">
-        <v>62644</v>
+        <v>62675</v>
       </c>
       <c r="P74" t="s">
-        <v>479</v>
+        <v>514</v>
       </c>
       <c r="Q74" t="s">
-        <v>480</v>
+        <v>515</v>
       </c>
       <c r="R74" t="s">
-        <v>481</v>
+        <v>516</v>
       </c>
       <c r="V74" t="s">
         <v>31</v>
@@ -5696,645 +5657,645 @@
     </row>
     <row r="75" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A75">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B75" t="s">
-        <v>482</v>
+        <v>517</v>
       </c>
       <c r="C75" t="s">
         <v>23</v>
       </c>
       <c r="H75" t="s">
-        <v>483</v>
+        <v>518</v>
       </c>
       <c r="K75" t="s">
-        <v>484</v>
+        <v>519</v>
       </c>
       <c r="M75" t="s">
-        <v>485</v>
+        <v>520</v>
       </c>
       <c r="N75" t="s">
         <v>27</v>
       </c>
       <c r="O75">
-        <v>62960</v>
+        <v>61231</v>
       </c>
       <c r="P75" t="s">
-        <v>486</v>
+        <v>521</v>
       </c>
       <c r="Q75" t="s">
-        <v>37</v>
+        <v>522</v>
       </c>
       <c r="R75" t="s">
-        <v>487</v>
+        <v>523</v>
       </c>
       <c r="V75" t="s">
-        <v>39</v>
+        <v>322</v>
       </c>
     </row>
     <row r="76" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A76">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B76" t="s">
-        <v>488</v>
+        <v>524</v>
       </c>
       <c r="C76" t="s">
         <v>23</v>
       </c>
       <c r="H76" t="s">
-        <v>489</v>
+        <v>525</v>
       </c>
       <c r="K76" t="s">
-        <v>490</v>
+        <v>526</v>
       </c>
       <c r="M76" t="s">
-        <v>491</v>
+        <v>527</v>
       </c>
       <c r="N76" t="s">
         <v>27</v>
       </c>
       <c r="O76">
-        <v>61455</v>
+        <v>62298</v>
       </c>
       <c r="P76" t="s">
-        <v>492</v>
+        <v>528</v>
       </c>
       <c r="Q76" t="s">
-        <v>493</v>
+        <v>529</v>
       </c>
       <c r="R76" t="s">
-        <v>494</v>
+        <v>530</v>
       </c>
       <c r="V76" t="s">
-        <v>270</v>
+        <v>531</v>
       </c>
     </row>
     <row r="77" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A77">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B77" t="s">
-        <v>495</v>
+        <v>532</v>
       </c>
       <c r="C77" t="s">
         <v>23</v>
       </c>
       <c r="H77" t="s">
-        <v>496</v>
+        <v>533</v>
       </c>
       <c r="K77" t="s">
-        <v>497</v>
+        <v>534</v>
       </c>
       <c r="M77" t="s">
-        <v>498</v>
+        <v>535</v>
       </c>
       <c r="N77" t="s">
         <v>27</v>
       </c>
       <c r="O77">
-        <v>60098</v>
+        <v>62049</v>
       </c>
       <c r="P77" t="s">
-        <v>499</v>
+        <v>536</v>
       </c>
       <c r="Q77" t="s">
-        <v>500</v>
+        <v>537</v>
       </c>
       <c r="R77" t="s">
-        <v>501</v>
+        <v>538</v>
       </c>
       <c r="V77" t="s">
-        <v>502</v>
+        <v>108</v>
       </c>
     </row>
     <row r="78" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A78">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B78" t="s">
-        <v>503</v>
+        <v>539</v>
       </c>
       <c r="C78" t="s">
         <v>23</v>
       </c>
       <c r="H78" t="s">
-        <v>504</v>
+        <v>540</v>
       </c>
       <c r="K78" t="s">
-        <v>505</v>
+        <v>541</v>
       </c>
       <c r="M78" t="s">
-        <v>506</v>
+        <v>542</v>
       </c>
       <c r="N78" t="s">
         <v>27</v>
       </c>
       <c r="O78">
-        <v>61701</v>
+        <v>62650</v>
       </c>
       <c r="P78" t="s">
-        <v>507</v>
+        <v>543</v>
       </c>
       <c r="Q78" t="s">
-        <v>508</v>
+        <v>544</v>
       </c>
       <c r="R78" t="s">
-        <v>509</v>
+        <v>545</v>
       </c>
       <c r="V78" t="s">
-        <v>255</v>
+        <v>283</v>
       </c>
     </row>
     <row r="79" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A79">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B79" t="s">
-        <v>510</v>
+        <v>546</v>
       </c>
       <c r="C79" t="s">
         <v>23</v>
       </c>
       <c r="H79" t="s">
-        <v>511</v>
+        <v>547</v>
       </c>
       <c r="K79" t="s">
-        <v>512</v>
+        <v>548</v>
       </c>
       <c r="M79" t="s">
-        <v>513</v>
+        <v>549</v>
       </c>
       <c r="N79" t="s">
         <v>27</v>
       </c>
       <c r="O79">
-        <v>62675</v>
+        <v>61951</v>
       </c>
       <c r="P79" t="s">
-        <v>514</v>
+        <v>550</v>
       </c>
       <c r="Q79" t="s">
-        <v>515</v>
+        <v>551</v>
       </c>
       <c r="R79" t="s">
-        <v>516</v>
+        <v>552</v>
       </c>
       <c r="V79" t="s">
-        <v>31</v>
+        <v>100</v>
       </c>
     </row>
     <row r="80" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A80">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B80" t="s">
-        <v>517</v>
+        <v>553</v>
       </c>
       <c r="C80" t="s">
         <v>23</v>
       </c>
       <c r="H80" t="s">
-        <v>518</v>
+        <v>554</v>
       </c>
       <c r="K80" t="s">
-        <v>519</v>
+        <v>555</v>
       </c>
       <c r="M80" t="s">
-        <v>520</v>
+        <v>556</v>
       </c>
       <c r="N80" t="s">
         <v>27</v>
       </c>
       <c r="O80">
-        <v>61231</v>
+        <v>61061</v>
       </c>
       <c r="P80" t="s">
-        <v>521</v>
+        <v>557</v>
       </c>
       <c r="Q80" t="s">
-        <v>522</v>
+        <v>423</v>
       </c>
       <c r="R80" t="s">
-        <v>523</v>
+        <v>558</v>
       </c>
       <c r="V80" t="s">
-        <v>322</v>
+        <v>425</v>
       </c>
     </row>
     <row r="81" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A81">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B81" t="s">
-        <v>524</v>
+        <v>559</v>
       </c>
       <c r="C81" t="s">
         <v>23</v>
       </c>
       <c r="H81" t="s">
-        <v>525</v>
+        <v>560</v>
       </c>
       <c r="K81" t="s">
-        <v>526</v>
+        <v>561</v>
       </c>
       <c r="M81" t="s">
-        <v>527</v>
+        <v>562</v>
       </c>
       <c r="N81" t="s">
         <v>27</v>
       </c>
       <c r="O81">
-        <v>62298</v>
+        <v>61602</v>
       </c>
       <c r="P81" t="s">
-        <v>528</v>
+        <v>562</v>
       </c>
       <c r="Q81" t="s">
-        <v>529</v>
+        <v>563</v>
       </c>
       <c r="R81" t="s">
-        <v>530</v>
+        <v>564</v>
       </c>
       <c r="V81" t="s">
-        <v>531</v>
+        <v>474</v>
       </c>
     </row>
     <row r="82" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A82">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B82" t="s">
-        <v>532</v>
+        <v>565</v>
       </c>
       <c r="C82" t="s">
         <v>23</v>
       </c>
       <c r="H82" t="s">
-        <v>533</v>
+        <v>566</v>
       </c>
       <c r="K82" t="s">
-        <v>534</v>
+        <v>567</v>
       </c>
       <c r="M82" t="s">
-        <v>535</v>
+        <v>568</v>
       </c>
       <c r="N82" t="s">
         <v>27</v>
       </c>
       <c r="O82">
-        <v>62049</v>
+        <v>62274</v>
       </c>
       <c r="P82" t="s">
-        <v>536</v>
-      </c>
-      <c r="Q82" t="s">
-        <v>537</v>
+        <v>569</v>
+      </c>
+      <c r="Q82" s="2" t="s">
+        <v>769</v>
       </c>
       <c r="R82" t="s">
-        <v>538</v>
+        <v>570</v>
       </c>
       <c r="V82" t="s">
-        <v>108</v>
+        <v>531</v>
       </c>
     </row>
     <row r="83" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A83">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B83" t="s">
-        <v>539</v>
+        <v>571</v>
       </c>
       <c r="C83" t="s">
         <v>23</v>
       </c>
       <c r="H83" t="s">
-        <v>540</v>
+        <v>572</v>
       </c>
       <c r="K83" t="s">
-        <v>541</v>
+        <v>573</v>
       </c>
       <c r="M83" t="s">
-        <v>542</v>
+        <v>574</v>
       </c>
       <c r="N83" t="s">
         <v>27</v>
       </c>
       <c r="O83">
-        <v>62650</v>
+        <v>61856</v>
       </c>
       <c r="P83" t="s">
-        <v>543</v>
+        <v>575</v>
       </c>
       <c r="Q83" t="s">
-        <v>544</v>
+        <v>576</v>
       </c>
       <c r="R83" t="s">
-        <v>545</v>
+        <v>577</v>
       </c>
       <c r="V83" t="s">
-        <v>283</v>
+        <v>100</v>
       </c>
     </row>
     <row r="84" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A84">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B84" t="s">
-        <v>546</v>
+        <v>578</v>
       </c>
       <c r="C84" t="s">
         <v>23</v>
       </c>
       <c r="H84" t="s">
-        <v>547</v>
+        <v>579</v>
       </c>
       <c r="K84" t="s">
-        <v>548</v>
+        <v>580</v>
       </c>
       <c r="M84" t="s">
-        <v>549</v>
+        <v>581</v>
       </c>
       <c r="N84" t="s">
         <v>27</v>
       </c>
       <c r="O84">
-        <v>61951</v>
+        <v>62363</v>
       </c>
       <c r="P84" t="s">
-        <v>550</v>
+        <v>582</v>
       </c>
       <c r="Q84" t="s">
-        <v>551</v>
+        <v>583</v>
       </c>
       <c r="R84" t="s">
-        <v>552</v>
+        <v>584</v>
       </c>
       <c r="V84" t="s">
-        <v>100</v>
+        <v>31</v>
       </c>
     </row>
     <row r="85" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A85">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B85" t="s">
-        <v>553</v>
+        <v>585</v>
       </c>
       <c r="C85" t="s">
         <v>23</v>
       </c>
       <c r="H85" t="s">
-        <v>554</v>
+        <v>586</v>
       </c>
       <c r="K85" t="s">
-        <v>555</v>
+        <v>587</v>
       </c>
       <c r="M85" t="s">
-        <v>556</v>
+        <v>588</v>
       </c>
       <c r="N85" t="s">
         <v>27</v>
       </c>
       <c r="O85">
-        <v>61061</v>
+        <v>62938</v>
       </c>
       <c r="P85" t="s">
-        <v>557</v>
+        <v>589</v>
       </c>
       <c r="Q85" t="s">
-        <v>423</v>
+        <v>37</v>
       </c>
       <c r="R85" t="s">
-        <v>558</v>
+        <v>590</v>
       </c>
       <c r="V85" t="s">
-        <v>425</v>
+        <v>39</v>
       </c>
     </row>
     <row r="86" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A86">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B86" t="s">
-        <v>559</v>
+        <v>591</v>
       </c>
       <c r="C86" t="s">
         <v>23</v>
       </c>
       <c r="H86" t="s">
-        <v>560</v>
+        <v>592</v>
       </c>
       <c r="K86" t="s">
-        <v>561</v>
+        <v>593</v>
       </c>
       <c r="M86" t="s">
-        <v>562</v>
+        <v>594</v>
       </c>
       <c r="N86" t="s">
         <v>27</v>
       </c>
       <c r="O86">
-        <v>61602</v>
+        <v>62963</v>
       </c>
       <c r="P86" t="s">
-        <v>562</v>
+        <v>595</v>
       </c>
       <c r="Q86" t="s">
-        <v>563</v>
+        <v>37</v>
       </c>
       <c r="R86" t="s">
-        <v>564</v>
+        <v>596</v>
       </c>
       <c r="V86" t="s">
-        <v>474</v>
+        <v>39</v>
       </c>
     </row>
     <row r="87" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A87">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B87" t="s">
-        <v>565</v>
+        <v>597</v>
       </c>
       <c r="C87" t="s">
         <v>23</v>
       </c>
       <c r="H87" t="s">
-        <v>566</v>
+        <v>598</v>
       </c>
       <c r="K87" t="s">
-        <v>567</v>
+        <v>599</v>
       </c>
       <c r="M87" t="s">
-        <v>568</v>
+        <v>600</v>
       </c>
       <c r="N87" t="s">
         <v>27</v>
       </c>
       <c r="O87">
-        <v>62274</v>
+        <v>61327</v>
       </c>
       <c r="P87" t="s">
-        <v>569</v>
-      </c>
-      <c r="Q87" s="2" t="s">
-        <v>769</v>
+        <v>601</v>
+      </c>
+      <c r="Q87" t="s">
+        <v>602</v>
       </c>
       <c r="R87" t="s">
-        <v>570</v>
+        <v>603</v>
       </c>
       <c r="V87" t="s">
-        <v>531</v>
+        <v>474</v>
       </c>
     </row>
     <row r="88" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A88">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B88" t="s">
-        <v>571</v>
+        <v>604</v>
       </c>
       <c r="C88" t="s">
         <v>23</v>
       </c>
       <c r="H88" t="s">
-        <v>572</v>
+        <v>605</v>
       </c>
       <c r="K88" t="s">
-        <v>573</v>
+        <v>606</v>
       </c>
       <c r="M88" t="s">
-        <v>574</v>
+        <v>607</v>
       </c>
       <c r="N88" t="s">
         <v>27</v>
       </c>
       <c r="O88">
-        <v>61856</v>
+        <v>62233</v>
       </c>
       <c r="P88" t="s">
-        <v>575</v>
+        <v>608</v>
       </c>
       <c r="Q88" t="s">
-        <v>576</v>
+        <v>609</v>
       </c>
       <c r="R88" t="s">
-        <v>577</v>
+        <v>610</v>
       </c>
       <c r="V88" t="s">
-        <v>100</v>
+        <v>531</v>
       </c>
     </row>
     <row r="89" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A89">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B89" t="s">
-        <v>578</v>
+        <v>611</v>
       </c>
       <c r="C89" t="s">
         <v>23</v>
       </c>
       <c r="H89" t="s">
-        <v>579</v>
+        <v>612</v>
       </c>
       <c r="K89" t="s">
-        <v>580</v>
+        <v>613</v>
       </c>
       <c r="M89" t="s">
-        <v>581</v>
+        <v>614</v>
       </c>
       <c r="N89" t="s">
         <v>27</v>
       </c>
       <c r="O89">
-        <v>62363</v>
+        <v>62450</v>
       </c>
       <c r="P89" t="s">
-        <v>582</v>
+        <v>615</v>
       </c>
       <c r="Q89" t="s">
-        <v>583</v>
+        <v>616</v>
       </c>
       <c r="R89" t="s">
-        <v>584</v>
+        <v>617</v>
       </c>
       <c r="V89" t="s">
-        <v>31</v>
+        <v>185</v>
       </c>
     </row>
     <row r="90" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A90">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B90" t="s">
-        <v>585</v>
+        <v>618</v>
       </c>
       <c r="C90" t="s">
         <v>23</v>
       </c>
       <c r="H90" t="s">
-        <v>586</v>
+        <v>619</v>
       </c>
       <c r="K90" t="s">
-        <v>587</v>
+        <v>620</v>
       </c>
       <c r="M90" t="s">
-        <v>588</v>
+        <v>621</v>
       </c>
       <c r="N90" t="s">
         <v>27</v>
       </c>
       <c r="O90">
-        <v>62938</v>
+        <v>61201</v>
       </c>
       <c r="P90" t="s">
-        <v>589</v>
+        <v>621</v>
       </c>
       <c r="Q90" t="s">
-        <v>37</v>
+        <v>622</v>
       </c>
       <c r="R90" t="s">
-        <v>590</v>
+        <v>623</v>
       </c>
       <c r="V90" t="s">
-        <v>39</v>
+        <v>322</v>
       </c>
     </row>
     <row r="91" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A91">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B91" t="s">
-        <v>591</v>
+        <v>624</v>
       </c>
       <c r="C91" t="s">
         <v>23</v>
       </c>
       <c r="H91" t="s">
-        <v>592</v>
+        <v>625</v>
       </c>
       <c r="K91" t="s">
-        <v>593</v>
+        <v>626</v>
       </c>
       <c r="M91" t="s">
-        <v>594</v>
+        <v>627</v>
       </c>
       <c r="N91" t="s">
         <v>27</v>
       </c>
       <c r="O91">
-        <v>62963</v>
+        <v>62946</v>
       </c>
       <c r="P91" t="s">
-        <v>595</v>
+        <v>628</v>
       </c>
       <c r="Q91" t="s">
         <v>37</v>
       </c>
       <c r="R91" t="s">
-        <v>596</v>
+        <v>629</v>
       </c>
       <c r="V91" t="s">
         <v>39</v>
@@ -6342,951 +6303,761 @@
     </row>
     <row r="92" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A92">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B92" t="s">
-        <v>597</v>
+        <v>630</v>
       </c>
       <c r="C92" t="s">
         <v>23</v>
       </c>
       <c r="H92" t="s">
-        <v>598</v>
+        <v>631</v>
       </c>
       <c r="K92" t="s">
-        <v>599</v>
+        <v>632</v>
       </c>
       <c r="M92" t="s">
-        <v>600</v>
+        <v>633</v>
       </c>
       <c r="N92" t="s">
         <v>27</v>
       </c>
       <c r="O92">
-        <v>61327</v>
+        <v>62701</v>
       </c>
       <c r="P92" t="s">
-        <v>601</v>
+        <v>634</v>
       </c>
       <c r="Q92" t="s">
-        <v>602</v>
+        <v>635</v>
       </c>
       <c r="R92" t="s">
-        <v>603</v>
+        <v>636</v>
       </c>
       <c r="V92" t="s">
-        <v>474</v>
+        <v>283</v>
       </c>
     </row>
     <row r="93" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A93">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B93" t="s">
-        <v>604</v>
+        <v>637</v>
       </c>
       <c r="C93" t="s">
         <v>23</v>
       </c>
       <c r="H93" t="s">
-        <v>605</v>
+        <v>638</v>
       </c>
       <c r="K93" t="s">
-        <v>606</v>
+        <v>639</v>
       </c>
       <c r="M93" t="s">
-        <v>607</v>
+        <v>640</v>
       </c>
       <c r="N93" t="s">
         <v>27</v>
       </c>
       <c r="O93">
-        <v>62233</v>
+        <v>62681</v>
       </c>
       <c r="P93" t="s">
-        <v>608</v>
+        <v>641</v>
       </c>
       <c r="Q93" t="s">
-        <v>609</v>
+        <v>642</v>
       </c>
       <c r="R93" t="s">
-        <v>610</v>
+        <v>643</v>
       </c>
       <c r="V93" t="s">
-        <v>531</v>
+        <v>31</v>
       </c>
     </row>
     <row r="94" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A94">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B94" t="s">
-        <v>611</v>
+        <v>644</v>
       </c>
       <c r="C94" t="s">
         <v>23</v>
       </c>
       <c r="H94" t="s">
-        <v>612</v>
+        <v>645</v>
       </c>
       <c r="K94" t="s">
-        <v>613</v>
+        <v>646</v>
       </c>
       <c r="M94" t="s">
-        <v>614</v>
+        <v>647</v>
       </c>
       <c r="N94" t="s">
         <v>27</v>
       </c>
       <c r="O94">
-        <v>62450</v>
+        <v>62694</v>
       </c>
       <c r="P94" t="s">
-        <v>615</v>
-      </c>
-      <c r="Q94" t="s">
-        <v>616</v>
+        <v>648</v>
+      </c>
+      <c r="Q94" s="2" t="s">
+        <v>765</v>
       </c>
       <c r="R94" t="s">
-        <v>617</v>
+        <v>649</v>
       </c>
       <c r="V94" t="s">
-        <v>185</v>
+        <v>283</v>
       </c>
     </row>
     <row r="95" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A95">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B95" t="s">
-        <v>618</v>
+        <v>650</v>
       </c>
       <c r="C95" t="s">
         <v>23</v>
       </c>
       <c r="H95" t="s">
-        <v>619</v>
+        <v>651</v>
       </c>
       <c r="K95" t="s">
-        <v>620</v>
+        <v>652</v>
       </c>
       <c r="M95" t="s">
-        <v>621</v>
+        <v>653</v>
       </c>
       <c r="N95" t="s">
         <v>27</v>
       </c>
       <c r="O95">
-        <v>61201</v>
+        <v>62565</v>
       </c>
       <c r="P95" t="s">
-        <v>621</v>
+        <v>654</v>
       </c>
       <c r="Q95" t="s">
-        <v>622</v>
+        <v>768</v>
       </c>
       <c r="R95" t="s">
-        <v>623</v>
+        <v>655</v>
       </c>
       <c r="V95" t="s">
-        <v>322</v>
+        <v>108</v>
       </c>
     </row>
     <row r="96" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A96">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B96" t="s">
-        <v>624</v>
+        <v>656</v>
       </c>
       <c r="C96" t="s">
         <v>23</v>
       </c>
       <c r="H96" t="s">
-        <v>625</v>
+        <v>657</v>
       </c>
       <c r="K96" t="s">
-        <v>626</v>
+        <v>658</v>
       </c>
       <c r="M96" t="s">
-        <v>627</v>
+        <v>659</v>
       </c>
       <c r="N96" t="s">
         <v>27</v>
       </c>
       <c r="O96">
-        <v>62946</v>
+        <v>62220</v>
       </c>
       <c r="P96" t="s">
-        <v>628</v>
+        <v>660</v>
       </c>
       <c r="Q96" t="s">
-        <v>37</v>
+        <v>661</v>
       </c>
       <c r="R96" t="s">
-        <v>629</v>
+        <v>662</v>
       </c>
       <c r="V96" t="s">
-        <v>39</v>
+        <v>663</v>
       </c>
     </row>
     <row r="97" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A97">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B97" t="s">
-        <v>630</v>
+        <v>664</v>
       </c>
       <c r="C97" t="s">
         <v>23</v>
       </c>
       <c r="H97" t="s">
-        <v>631</v>
+        <v>665</v>
       </c>
       <c r="K97" t="s">
-        <v>632</v>
+        <v>666</v>
       </c>
       <c r="M97" t="s">
-        <v>633</v>
+        <v>667</v>
       </c>
       <c r="N97" t="s">
         <v>27</v>
       </c>
       <c r="O97">
-        <v>62701</v>
+        <v>61483</v>
       </c>
       <c r="P97" t="s">
-        <v>634</v>
+        <v>668</v>
       </c>
       <c r="Q97" t="s">
-        <v>635</v>
+        <v>669</v>
       </c>
       <c r="R97" t="s">
-        <v>636</v>
+        <v>670</v>
       </c>
       <c r="V97" t="s">
-        <v>283</v>
+        <v>474</v>
       </c>
     </row>
     <row r="98" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A98">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B98" t="s">
-        <v>637</v>
+        <v>671</v>
       </c>
       <c r="C98" t="s">
         <v>23</v>
       </c>
       <c r="H98" t="s">
-        <v>638</v>
+        <v>672</v>
       </c>
       <c r="K98" t="s">
-        <v>639</v>
+        <v>673</v>
       </c>
       <c r="M98" t="s">
-        <v>640</v>
+        <v>674</v>
       </c>
       <c r="N98" t="s">
         <v>27</v>
       </c>
       <c r="O98">
-        <v>62681</v>
+        <v>61032</v>
       </c>
       <c r="P98" t="s">
-        <v>641</v>
+        <v>675</v>
       </c>
       <c r="Q98" t="s">
-        <v>642</v>
+        <v>423</v>
       </c>
       <c r="R98" t="s">
-        <v>643</v>
+        <v>676</v>
       </c>
       <c r="V98" t="s">
-        <v>31</v>
+        <v>425</v>
       </c>
     </row>
     <row r="99" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A99">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B99" t="s">
-        <v>644</v>
+        <v>677</v>
       </c>
       <c r="C99" t="s">
         <v>23</v>
       </c>
       <c r="H99" t="s">
-        <v>645</v>
+        <v>678</v>
       </c>
       <c r="K99" t="s">
-        <v>646</v>
+        <v>679</v>
       </c>
       <c r="M99" t="s">
-        <v>647</v>
+        <v>680</v>
       </c>
       <c r="N99" t="s">
         <v>27</v>
       </c>
       <c r="O99">
-        <v>62694</v>
+        <v>61554</v>
       </c>
       <c r="P99" t="s">
-        <v>648</v>
-      </c>
-      <c r="Q99" s="2" t="s">
-        <v>765</v>
+        <v>681</v>
+      </c>
+      <c r="Q99" t="s">
+        <v>682</v>
       </c>
       <c r="R99" t="s">
-        <v>649</v>
+        <v>683</v>
       </c>
       <c r="V99" t="s">
-        <v>283</v>
+        <v>474</v>
       </c>
     </row>
     <row r="100" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A100">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B100" t="s">
-        <v>650</v>
+        <v>684</v>
       </c>
       <c r="C100" t="s">
         <v>23</v>
       </c>
       <c r="H100" t="s">
-        <v>651</v>
+        <v>685</v>
       </c>
       <c r="K100" t="s">
-        <v>652</v>
+        <v>686</v>
       </c>
       <c r="M100" t="s">
-        <v>653</v>
+        <v>687</v>
       </c>
       <c r="N100" t="s">
         <v>27</v>
       </c>
       <c r="O100">
-        <v>62565</v>
+        <v>62952</v>
       </c>
       <c r="P100" t="s">
-        <v>654</v>
+        <v>688</v>
       </c>
       <c r="Q100" t="s">
-        <v>768</v>
+        <v>689</v>
       </c>
       <c r="R100" t="s">
-        <v>655</v>
+        <v>690</v>
       </c>
       <c r="V100" t="s">
-        <v>108</v>
+        <v>39</v>
       </c>
     </row>
     <row r="101" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A101">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B101" t="s">
-        <v>656</v>
+        <v>691</v>
       </c>
       <c r="C101" t="s">
         <v>23</v>
       </c>
       <c r="H101" t="s">
-        <v>657</v>
+        <v>692</v>
       </c>
       <c r="K101" t="s">
-        <v>658</v>
+        <v>693</v>
       </c>
       <c r="M101" t="s">
-        <v>659</v>
+        <v>694</v>
       </c>
       <c r="N101" t="s">
         <v>27</v>
       </c>
       <c r="O101">
-        <v>62220</v>
+        <v>61832</v>
       </c>
       <c r="P101" t="s">
-        <v>660</v>
+        <v>695</v>
       </c>
       <c r="Q101" t="s">
-        <v>661</v>
+        <v>696</v>
       </c>
       <c r="R101" t="s">
-        <v>662</v>
+        <v>697</v>
       </c>
       <c r="V101" t="s">
-        <v>663</v>
+        <v>116</v>
       </c>
     </row>
     <row r="102" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A102">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B102" t="s">
-        <v>664</v>
+        <v>698</v>
       </c>
       <c r="C102" t="s">
         <v>23</v>
       </c>
       <c r="H102" t="s">
-        <v>665</v>
+        <v>699</v>
       </c>
       <c r="K102" t="s">
-        <v>666</v>
+        <v>700</v>
       </c>
       <c r="M102" t="s">
-        <v>667</v>
+        <v>701</v>
       </c>
       <c r="N102" t="s">
         <v>27</v>
       </c>
       <c r="O102">
-        <v>61483</v>
+        <v>62863</v>
       </c>
       <c r="P102" t="s">
-        <v>668</v>
+        <v>702</v>
       </c>
       <c r="Q102" t="s">
-        <v>669</v>
+        <v>183</v>
       </c>
       <c r="R102" t="s">
-        <v>670</v>
+        <v>703</v>
       </c>
       <c r="V102" t="s">
-        <v>474</v>
+        <v>185</v>
       </c>
     </row>
     <row r="103" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A103">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B103" t="s">
-        <v>671</v>
+        <v>704</v>
       </c>
       <c r="C103" t="s">
         <v>23</v>
       </c>
       <c r="H103" t="s">
-        <v>672</v>
+        <v>298</v>
       </c>
       <c r="K103" t="s">
-        <v>673</v>
+        <v>705</v>
       </c>
       <c r="M103" t="s">
-        <v>674</v>
+        <v>706</v>
       </c>
       <c r="N103" t="s">
         <v>27</v>
       </c>
       <c r="O103">
-        <v>61032</v>
+        <v>61462</v>
       </c>
       <c r="P103" t="s">
-        <v>675</v>
+        <v>707</v>
       </c>
       <c r="Q103" t="s">
-        <v>423</v>
+        <v>708</v>
       </c>
       <c r="R103" t="s">
-        <v>676</v>
+        <v>709</v>
       </c>
       <c r="V103" t="s">
-        <v>425</v>
+        <v>270</v>
       </c>
     </row>
     <row r="104" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A104">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B104" t="s">
-        <v>677</v>
+        <v>710</v>
       </c>
       <c r="C104" t="s">
         <v>23</v>
       </c>
       <c r="H104" t="s">
-        <v>678</v>
+        <v>711</v>
       </c>
       <c r="K104" t="s">
-        <v>679</v>
+        <v>712</v>
       </c>
       <c r="M104" t="s">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="N104" t="s">
         <v>27</v>
       </c>
       <c r="O104">
-        <v>61554</v>
+        <v>62263</v>
       </c>
       <c r="P104" t="s">
-        <v>681</v>
+        <v>714</v>
       </c>
       <c r="Q104" t="s">
-        <v>682</v>
+        <v>715</v>
       </c>
       <c r="R104" t="s">
-        <v>683</v>
+        <v>716</v>
       </c>
       <c r="V104" t="s">
-        <v>474</v>
+        <v>531</v>
       </c>
     </row>
     <row r="105" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A105">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B105" t="s">
-        <v>684</v>
+        <v>717</v>
       </c>
       <c r="C105" t="s">
         <v>23</v>
       </c>
       <c r="H105" t="s">
-        <v>685</v>
+        <v>718</v>
       </c>
       <c r="K105" t="s">
-        <v>686</v>
+        <v>719</v>
       </c>
       <c r="M105" t="s">
-        <v>687</v>
+        <v>720</v>
       </c>
       <c r="N105" t="s">
         <v>27</v>
       </c>
       <c r="O105">
-        <v>62952</v>
+        <v>62837</v>
       </c>
       <c r="P105" t="s">
-        <v>688</v>
+        <v>721</v>
       </c>
       <c r="Q105" t="s">
-        <v>689</v>
+        <v>722</v>
       </c>
       <c r="R105" t="s">
-        <v>690</v>
+        <v>723</v>
       </c>
       <c r="V105" t="s">
-        <v>39</v>
+        <v>185</v>
       </c>
     </row>
     <row r="106" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A106">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B106" t="s">
-        <v>691</v>
+        <v>724</v>
       </c>
       <c r="C106" t="s">
         <v>23</v>
       </c>
       <c r="H106" t="s">
-        <v>692</v>
+        <v>725</v>
       </c>
       <c r="K106" t="s">
-        <v>693</v>
+        <v>726</v>
       </c>
       <c r="M106" t="s">
-        <v>694</v>
+        <v>727</v>
       </c>
       <c r="N106" t="s">
         <v>27</v>
       </c>
       <c r="O106">
-        <v>61832</v>
+        <v>62821</v>
       </c>
       <c r="P106" t="s">
-        <v>695</v>
+        <v>728</v>
       </c>
       <c r="Q106" t="s">
-        <v>696</v>
+        <v>183</v>
       </c>
       <c r="R106" t="s">
-        <v>697</v>
+        <v>729</v>
       </c>
       <c r="V106" t="s">
-        <v>116</v>
+        <v>185</v>
       </c>
     </row>
     <row r="107" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A107">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B107" t="s">
-        <v>698</v>
+        <v>730</v>
       </c>
       <c r="C107" t="s">
         <v>23</v>
       </c>
       <c r="H107" t="s">
-        <v>699</v>
+        <v>731</v>
       </c>
       <c r="K107" t="s">
-        <v>700</v>
+        <v>732</v>
       </c>
       <c r="M107" t="s">
-        <v>701</v>
+        <v>733</v>
       </c>
       <c r="N107" t="s">
         <v>27</v>
       </c>
       <c r="O107">
-        <v>62863</v>
+        <v>61270</v>
       </c>
       <c r="P107" t="s">
-        <v>702</v>
+        <v>734</v>
       </c>
       <c r="Q107" t="s">
-        <v>183</v>
+        <v>735</v>
       </c>
       <c r="R107" t="s">
-        <v>703</v>
+        <v>736</v>
       </c>
       <c r="V107" t="s">
-        <v>185</v>
+        <v>322</v>
       </c>
     </row>
     <row r="108" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A108">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B108" t="s">
-        <v>704</v>
+        <v>737</v>
       </c>
       <c r="C108" t="s">
         <v>23</v>
       </c>
       <c r="H108" t="s">
-        <v>298</v>
+        <v>738</v>
       </c>
       <c r="K108" t="s">
-        <v>705</v>
+        <v>739</v>
       </c>
       <c r="M108" t="s">
-        <v>706</v>
+        <v>740</v>
       </c>
       <c r="N108" t="s">
         <v>27</v>
       </c>
       <c r="O108">
-        <v>61462</v>
+        <v>60432</v>
       </c>
       <c r="P108" t="s">
-        <v>707</v>
+        <v>741</v>
       </c>
       <c r="Q108" t="s">
-        <v>708</v>
+        <v>742</v>
       </c>
       <c r="R108" t="s">
-        <v>709</v>
+        <v>743</v>
       </c>
       <c r="V108" t="s">
-        <v>270</v>
+        <v>744</v>
       </c>
     </row>
     <row r="109" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A109">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B109" t="s">
-        <v>710</v>
+        <v>745</v>
       </c>
       <c r="C109" t="s">
         <v>23</v>
       </c>
       <c r="H109" t="s">
-        <v>711</v>
+        <v>746</v>
       </c>
       <c r="K109" t="s">
-        <v>712</v>
+        <v>747</v>
       </c>
       <c r="M109" t="s">
-        <v>713</v>
+        <v>465</v>
       </c>
       <c r="N109" t="s">
         <v>27</v>
       </c>
       <c r="O109">
-        <v>62263</v>
+        <v>62959</v>
       </c>
       <c r="P109" t="s">
-        <v>714</v>
+        <v>748</v>
       </c>
       <c r="Q109" t="s">
-        <v>715</v>
+        <v>37</v>
       </c>
       <c r="R109" t="s">
-        <v>716</v>
+        <v>749</v>
       </c>
       <c r="V109" t="s">
-        <v>531</v>
+        <v>39</v>
       </c>
     </row>
     <row r="110" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A110">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B110" t="s">
-        <v>717</v>
+        <v>750</v>
       </c>
       <c r="C110" t="s">
         <v>23</v>
       </c>
       <c r="H110" t="s">
-        <v>718</v>
+        <v>751</v>
       </c>
       <c r="K110" t="s">
-        <v>719</v>
+        <v>752</v>
       </c>
       <c r="M110" t="s">
-        <v>720</v>
+        <v>753</v>
       </c>
       <c r="N110" t="s">
         <v>27</v>
       </c>
       <c r="O110">
-        <v>62837</v>
+        <v>61101</v>
       </c>
       <c r="P110" t="s">
-        <v>721</v>
+        <v>754</v>
       </c>
       <c r="Q110" t="s">
-        <v>722</v>
+        <v>755</v>
       </c>
       <c r="R110" t="s">
-        <v>723</v>
+        <v>756</v>
       </c>
       <c r="V110" t="s">
-        <v>185</v>
+        <v>55</v>
       </c>
     </row>
     <row r="111" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A111">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B111" t="s">
-        <v>724</v>
+        <v>757</v>
       </c>
       <c r="C111" t="s">
         <v>23</v>
       </c>
       <c r="H111" t="s">
-        <v>725</v>
+        <v>758</v>
       </c>
       <c r="K111" t="s">
-        <v>726</v>
+        <v>759</v>
       </c>
       <c r="M111" t="s">
-        <v>727</v>
+        <v>760</v>
       </c>
       <c r="N111" t="s">
         <v>27</v>
       </c>
       <c r="O111">
-        <v>62821</v>
+        <v>61530</v>
       </c>
       <c r="P111" t="s">
-        <v>728</v>
+        <v>761</v>
       </c>
       <c r="Q111" t="s">
-        <v>183</v>
+        <v>762</v>
       </c>
       <c r="R111" t="s">
-        <v>729</v>
+        <v>763</v>
       </c>
       <c r="V111" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A112">
-        <v>98</v>
-      </c>
-      <c r="B112" t="s">
-        <v>730</v>
-      </c>
-      <c r="C112" t="s">
-        <v>23</v>
-      </c>
-      <c r="H112" t="s">
-        <v>731</v>
-      </c>
-      <c r="K112" t="s">
-        <v>732</v>
-      </c>
-      <c r="M112" t="s">
-        <v>733</v>
-      </c>
-      <c r="N112" t="s">
-        <v>27</v>
-      </c>
-      <c r="O112">
-        <v>61270</v>
-      </c>
-      <c r="P112" t="s">
-        <v>734</v>
-      </c>
-      <c r="Q112" t="s">
-        <v>735</v>
-      </c>
-      <c r="R112" t="s">
-        <v>736</v>
-      </c>
-      <c r="V112" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="113" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A113">
-        <v>99</v>
-      </c>
-      <c r="B113" t="s">
-        <v>737</v>
-      </c>
-      <c r="C113" t="s">
-        <v>23</v>
-      </c>
-      <c r="H113" t="s">
-        <v>738</v>
-      </c>
-      <c r="K113" t="s">
-        <v>739</v>
-      </c>
-      <c r="M113" t="s">
-        <v>740</v>
-      </c>
-      <c r="N113" t="s">
-        <v>27</v>
-      </c>
-      <c r="O113">
-        <v>60432</v>
-      </c>
-      <c r="P113" t="s">
-        <v>741</v>
-      </c>
-      <c r="Q113" t="s">
-        <v>742</v>
-      </c>
-      <c r="R113" t="s">
-        <v>743</v>
-      </c>
-      <c r="V113" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="114" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A114">
-        <v>100</v>
-      </c>
-      <c r="B114" t="s">
-        <v>745</v>
-      </c>
-      <c r="C114" t="s">
-        <v>23</v>
-      </c>
-      <c r="H114" t="s">
-        <v>746</v>
-      </c>
-      <c r="K114" t="s">
-        <v>747</v>
-      </c>
-      <c r="M114" t="s">
-        <v>465</v>
-      </c>
-      <c r="N114" t="s">
-        <v>27</v>
-      </c>
-      <c r="O114">
-        <v>62959</v>
-      </c>
-      <c r="P114" t="s">
-        <v>748</v>
-      </c>
-      <c r="Q114" t="s">
-        <v>37</v>
-      </c>
-      <c r="R114" t="s">
-        <v>749</v>
-      </c>
-      <c r="V114" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A115">
-        <v>101</v>
-      </c>
-      <c r="B115" t="s">
-        <v>750</v>
-      </c>
-      <c r="C115" t="s">
-        <v>23</v>
-      </c>
-      <c r="H115" t="s">
-        <v>751</v>
-      </c>
-      <c r="K115" t="s">
-        <v>752</v>
-      </c>
-      <c r="M115" t="s">
-        <v>753</v>
-      </c>
-      <c r="N115" t="s">
-        <v>27</v>
-      </c>
-      <c r="O115">
-        <v>61101</v>
-      </c>
-      <c r="P115" t="s">
-        <v>754</v>
-      </c>
-      <c r="Q115" t="s">
-        <v>755</v>
-      </c>
-      <c r="R115" t="s">
-        <v>756</v>
-      </c>
-      <c r="V115" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="116" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A116">
-        <v>102</v>
-      </c>
-      <c r="B116" t="s">
-        <v>757</v>
-      </c>
-      <c r="C116" t="s">
-        <v>23</v>
-      </c>
-      <c r="H116" t="s">
-        <v>758</v>
-      </c>
-      <c r="K116" t="s">
-        <v>759</v>
-      </c>
-      <c r="M116" t="s">
-        <v>760</v>
-      </c>
-      <c r="N116" t="s">
-        <v>27</v>
-      </c>
-      <c r="O116">
-        <v>61530</v>
-      </c>
-      <c r="P116" t="s">
-        <v>761</v>
-      </c>
-      <c r="Q116" t="s">
-        <v>762</v>
-      </c>
-      <c r="R116" t="s">
-        <v>763</v>
-      </c>
-      <c r="V116" t="s">
         <v>255</v>
       </c>
     </row>
@@ -7297,9 +7068,9 @@
     <hyperlink ref="Q45" r:id="rId3" xr:uid="{E8701583-F1BF-4A71-A500-C737411446E5}"/>
     <hyperlink ref="Q44" r:id="rId4" xr:uid="{9BB64827-CBE0-4F72-88A8-10DFB32413E9}"/>
     <hyperlink ref="Q49" r:id="rId5" xr:uid="{231A7501-BA49-418B-817D-98BB18CD74C8}"/>
-    <hyperlink ref="Q65" r:id="rId6" xr:uid="{4B7E1D46-47BF-4923-887D-F0D311096F3B}"/>
-    <hyperlink ref="Q87" r:id="rId7" xr:uid="{968EC501-FFBE-489E-849D-C2279F57E36E}"/>
-    <hyperlink ref="Q99" r:id="rId8" xr:uid="{EDF05CEF-DF2C-4746-B08F-B2D45EF1CA5F}"/>
+    <hyperlink ref="Q60" r:id="rId6" xr:uid="{4B7E1D46-47BF-4923-887D-F0D311096F3B}"/>
+    <hyperlink ref="Q82" r:id="rId7" xr:uid="{968EC501-FFBE-489E-849D-C2279F57E36E}"/>
+    <hyperlink ref="Q94" r:id="rId8" xr:uid="{EDF05CEF-DF2C-4746-B08F-B2D45EF1CA5F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>